<commit_message>
Atualiza dados - 09/04/2026  8:32
</commit_message>
<xml_diff>
--- a/public/saldo_por_gestor.xlsx
+++ b/public/saldo_por_gestor.xlsx
@@ -397,13 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D92"/>
-  <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -455,10 +449,10 @@
         <v>Claudio Bispo Dos Santos</v>
       </c>
       <c r="C4" t="str">
-        <v>-14h22min</v>
+        <v>-114h46min</v>
       </c>
       <c r="D4">
-        <v>-862</v>
+        <v>-6886</v>
       </c>
     </row>
     <row r="5">
@@ -567,10 +561,10 @@
         <v>Paulo Cesar Da Silva Santos Junior</v>
       </c>
       <c r="C12" t="str">
-        <v>-27h</v>
+        <v>-52h48min</v>
       </c>
       <c r="D12">
-        <v>-1620</v>
+        <v>-3168</v>
       </c>
     </row>
     <row r="13">
@@ -592,13 +586,13 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B14" t="str">
-        <v>Rosilene Martins Da Silva</v>
+        <v>Robéria Gilo Da Silva</v>
       </c>
       <c r="C14" t="str">
-        <v>-35h16min</v>
+        <v>-47h35min</v>
       </c>
       <c r="D14">
-        <v>-2116</v>
+        <v>-2855</v>
       </c>
     </row>
     <row r="15">
@@ -606,13 +600,13 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B15" t="str">
-        <v>Thalys Gomes Dos Santos</v>
+        <v>Rosilene Martins Da Silva</v>
       </c>
       <c r="C15" t="str">
-        <v>-42h4min</v>
+        <v>-35h16min</v>
       </c>
       <c r="D15">
-        <v>-2524</v>
+        <v>-2116</v>
       </c>
     </row>
     <row r="16">
@@ -620,27 +614,27 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B16" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Thalys Gomes Dos Santos</v>
       </c>
       <c r="C16" t="str">
-        <v>+30h18min</v>
+        <v>-42h4min</v>
       </c>
       <c r="D16">
-        <v>1818</v>
+        <v>-2524</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B17" t="str">
-        <v>Ane Caroline Pereira marter</v>
+        <v>Yuri Castro Gomes</v>
       </c>
       <c r="C17" t="str">
-        <v>+11h23min</v>
+        <v>+30h18min</v>
       </c>
       <c r="D17">
-        <v>683</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="18">
@@ -648,13 +642,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B18" t="str">
-        <v>Anny Karoline Andrade Santos</v>
+        <v>Ane Caroline Pereira marter</v>
       </c>
       <c r="C18" t="str">
-        <v>-44h19min</v>
+        <v>+11h23min</v>
       </c>
       <c r="D18">
-        <v>-2659</v>
+        <v>683</v>
       </c>
     </row>
     <row r="19">
@@ -662,13 +656,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B19" t="str">
-        <v>Kamilla Santos da Silva</v>
+        <v>Anny Karoline Andrade Santos</v>
       </c>
       <c r="C19" t="str">
-        <v>-23h12min</v>
+        <v>-44h19min</v>
       </c>
       <c r="D19">
-        <v>-1392</v>
+        <v>-2659</v>
       </c>
     </row>
     <row r="20">
@@ -676,13 +670,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B20" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Kamilla Santos da Silva</v>
       </c>
       <c r="C20" t="str">
-        <v>+20h3min</v>
+        <v>-23h12min</v>
       </c>
       <c r="D20">
-        <v>1203</v>
+        <v>-1392</v>
       </c>
     </row>
     <row r="21">
@@ -690,13 +684,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B21" t="str">
-        <v>Sandra da Conceição Freitas</v>
+        <v>Maria Jeane da Silva Santos</v>
       </c>
       <c r="C21" t="str">
-        <v>+5h6min</v>
+        <v>+2h59min</v>
       </c>
       <c r="D21">
-        <v>306</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22">
@@ -704,55 +698,55 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B22" t="str">
-        <v>Thamires Emanuelle da Silva</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
       <c r="C22" t="str">
-        <v>-2h26min</v>
+        <v>+20h3min</v>
       </c>
       <c r="D22">
-        <v>-146</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B23" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Sandra da Conceição Freitas</v>
       </c>
       <c r="C23" t="str">
-        <v>-61h48min</v>
+        <v>+5h6min</v>
       </c>
       <c r="D23">
-        <v>-3708</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B24" t="str">
-        <v>Ana Luiza Dos Santos</v>
+        <v>Thamires Emanuelle da Silva</v>
       </c>
       <c r="C24" t="str">
-        <v>-29h7min</v>
+        <v>-2h26min</v>
       </c>
       <c r="D24">
-        <v>-1747</v>
+        <v>-146</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B25" t="str">
-        <v>Emanoelle Feitosa Vieira Santos</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="C25" t="str">
-        <v>-31h57min</v>
+        <v>-61h48min</v>
       </c>
       <c r="D25">
-        <v>-1917</v>
+        <v>-3708</v>
       </c>
     </row>
     <row r="26">
@@ -760,13 +754,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B26" t="str">
-        <v>Gessica Aparecida Dos Santos</v>
+        <v>Ana Luiza Dos Santos</v>
       </c>
       <c r="C26" t="str">
-        <v>-96h27min</v>
+        <v>-76h31min</v>
       </c>
       <c r="D26">
-        <v>-5787</v>
+        <v>-4591</v>
       </c>
     </row>
     <row r="27">
@@ -774,13 +768,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B27" t="str">
-        <v>Giselle Dos Santos Roberto</v>
+        <v>Emanoelle Feitosa Vieira Santos</v>
       </c>
       <c r="C27" t="str">
-        <v>-47h7min</v>
+        <v>-31h57min</v>
       </c>
       <c r="D27">
-        <v>-2827</v>
+        <v>-1917</v>
       </c>
     </row>
     <row r="28">
@@ -788,13 +782,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B28" t="str">
-        <v>Kauanne Iwashita Da Silva</v>
+        <v>Gessica Aparecida Dos Santos</v>
       </c>
       <c r="C28" t="str">
-        <v>-32h13min</v>
+        <v>-122h57min</v>
       </c>
       <c r="D28">
-        <v>-1933</v>
+        <v>-7377</v>
       </c>
     </row>
     <row r="29">
@@ -802,13 +796,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B29" t="str">
-        <v>Laís Manuelle Santos Pereira</v>
+        <v>Giselle Dos Santos Roberto</v>
       </c>
       <c r="C29" t="str">
-        <v>-16h57min</v>
+        <v>-47h7min</v>
       </c>
       <c r="D29">
-        <v>-1017</v>
+        <v>-2827</v>
       </c>
     </row>
     <row r="30">
@@ -816,13 +810,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B30" t="str">
-        <v>Leticia Seixas Santos</v>
+        <v>Kauanne Iwashita Da Silva</v>
       </c>
       <c r="C30" t="str">
-        <v>-16h41min</v>
+        <v>-224h49min</v>
       </c>
       <c r="D30">
-        <v>-1001</v>
+        <v>-13489</v>
       </c>
     </row>
     <row r="31">
@@ -830,13 +824,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B31" t="str">
-        <v>Luciene Da Silva Nascimento</v>
+        <v>Laís Manuelle Santos Pereira</v>
       </c>
       <c r="C31" t="str">
-        <v>-39h36min</v>
+        <v>-16h57min</v>
       </c>
       <c r="D31">
-        <v>-2376</v>
+        <v>-1017</v>
       </c>
     </row>
     <row r="32">
@@ -844,13 +838,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B32" t="str">
-        <v>Natali de Souza Gonzaga</v>
+        <v>Leticia Seixas Santos</v>
       </c>
       <c r="C32" t="str">
-        <v>-58h39min</v>
+        <v>-12h19min</v>
       </c>
       <c r="D32">
-        <v>-3519</v>
+        <v>-739</v>
       </c>
     </row>
     <row r="33">
@@ -858,13 +852,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B33" t="str">
-        <v>Nathalia Vieira Lima</v>
+        <v>Luciene Da Silva Nascimento</v>
       </c>
       <c r="C33" t="str">
-        <v>-73h26min</v>
+        <v>-10h35min</v>
       </c>
       <c r="D33">
-        <v>-4406</v>
+        <v>-635</v>
       </c>
     </row>
     <row r="34">
@@ -872,41 +866,41 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B34" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Natali de Souza Gonzaga</v>
       </c>
       <c r="C34" t="str">
-        <v>+0h</v>
+        <v>-58h39min</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>-3519</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B35" t="str">
-        <v>Fabia Batista da Silva</v>
+        <v>Nathalia Vieira Lima</v>
       </c>
       <c r="C35" t="str">
-        <v>-26h19min</v>
+        <v>-73h4min</v>
       </c>
       <c r="D35">
-        <v>-1579</v>
+        <v>-4384</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B36" t="str">
-        <v>Gessyca Nayara Rocha Santos</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
       <c r="C36" t="str">
-        <v>-43h12min</v>
+        <v>-188h</v>
       </c>
       <c r="D36">
-        <v>-2592</v>
+        <v>-11280</v>
       </c>
     </row>
     <row r="37">
@@ -914,13 +908,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B37" t="str">
-        <v>Jaine Mariana Rodrigues Mendonça</v>
+        <v>Fabia Batista da Silva</v>
       </c>
       <c r="C37" t="str">
-        <v>-3h42min</v>
+        <v>-26h19min</v>
       </c>
       <c r="D37">
-        <v>-222</v>
+        <v>-1579</v>
       </c>
     </row>
     <row r="38">
@@ -928,13 +922,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B38" t="str">
-        <v>Karine Celestino Evangelista dos Santos</v>
+        <v>Gessyca Nayara Rocha Santos</v>
       </c>
       <c r="C38" t="str">
-        <v>-12h53min</v>
+        <v>-156h27min</v>
       </c>
       <c r="D38">
-        <v>-773</v>
+        <v>-9387</v>
       </c>
     </row>
     <row r="39">
@@ -942,41 +936,41 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B39" t="str">
-        <v>Maria Tatiane Oliveira Santos</v>
+        <v>Jaine Mariana Rodrigues Mendonça</v>
       </c>
       <c r="C39" t="str">
-        <v>-52h59min</v>
+        <v>-3h42min</v>
       </c>
       <c r="D39">
-        <v>-3179</v>
+        <v>-222</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B40" t="str">
-        <v>Bruna Candido de Lima</v>
+        <v>Karine Celestino Evangelista dos Santos</v>
       </c>
       <c r="C40" t="str">
-        <v>+3h37min</v>
+        <v>-12h53min</v>
       </c>
       <c r="D40">
-        <v>217</v>
+        <v>-773</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B41" t="str">
-        <v>Camilla Emanuelle Lopes de Almeida</v>
+        <v>Maria Tatiane Oliveira Santos</v>
       </c>
       <c r="C41" t="str">
-        <v>-9h21min</v>
+        <v>-65h47min</v>
       </c>
       <c r="D41">
-        <v>-561</v>
+        <v>-3947</v>
       </c>
     </row>
     <row r="42">
@@ -984,13 +978,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B42" t="str">
-        <v>Danielle Dos Santos Silva</v>
+        <v>Bruna Candido de Lima</v>
       </c>
       <c r="C42" t="str">
-        <v>-26h55min</v>
+        <v>+3h37min</v>
       </c>
       <c r="D42">
-        <v>-1615</v>
+        <v>217</v>
       </c>
     </row>
     <row r="43">
@@ -998,13 +992,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B43" t="str">
-        <v>Edna Lopes Da Silva</v>
+        <v>Camilla Emanuelle Lopes de Almeida</v>
       </c>
       <c r="C43" t="str">
-        <v>+12h</v>
+        <v>-9h21min</v>
       </c>
       <c r="D43">
-        <v>720</v>
+        <v>-561</v>
       </c>
     </row>
     <row r="44">
@@ -1012,13 +1006,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B44" t="str">
-        <v>Jordelle Meygre Costa De Oliveira</v>
+        <v>Danielle Dos Santos Silva</v>
       </c>
       <c r="C44" t="str">
-        <v>+25h47min</v>
+        <v>-0h43min</v>
       </c>
       <c r="D44">
-        <v>1547</v>
+        <v>-43</v>
       </c>
     </row>
     <row r="45">
@@ -1026,13 +1020,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B45" t="str">
-        <v>Lays da Silva Vieira</v>
+        <v>Edna Lopes Da Silva</v>
       </c>
       <c r="C45" t="str">
-        <v>+0h27min</v>
+        <v>+173h46min</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>10426</v>
       </c>
     </row>
     <row r="46">
@@ -1040,13 +1034,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B46" t="str">
-        <v>Luan Santos de Oliveira</v>
+        <v>Jordelle Meygre Costa De Oliveira</v>
       </c>
       <c r="C46" t="str">
-        <v>+9h26min</v>
+        <v>+51h49min</v>
       </c>
       <c r="D46">
-        <v>566</v>
+        <v>3109</v>
       </c>
     </row>
     <row r="47">
@@ -1054,13 +1048,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B47" t="str">
-        <v>Maria Victoria Souza Araujo Ferro</v>
+        <v>Lays da Silva Vieira</v>
       </c>
       <c r="C47" t="str">
-        <v>-29h32min</v>
+        <v>+0h27min</v>
       </c>
       <c r="D47">
-        <v>-1772</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48">
@@ -1068,13 +1062,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B48" t="str">
-        <v>Marília Alice dos Santos Silva</v>
+        <v>Luan Santos de Oliveira</v>
       </c>
       <c r="C48" t="str">
-        <v>+1h21min</v>
+        <v>+9h26min</v>
       </c>
       <c r="D48">
-        <v>81</v>
+        <v>566</v>
       </c>
     </row>
     <row r="49">
@@ -1082,13 +1076,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B49" t="str">
-        <v>Raquele Fragoso Da Silva</v>
+        <v>Maria Victoria Souza Araujo Ferro</v>
       </c>
       <c r="C49" t="str">
-        <v>-35h27min</v>
+        <v>-29h32min</v>
       </c>
       <c r="D49">
-        <v>-2127</v>
+        <v>-1772</v>
       </c>
     </row>
     <row r="50">
@@ -1096,41 +1090,41 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B50" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Marília Alice dos Santos Silva</v>
       </c>
       <c r="C50" t="str">
-        <v>-2h59min</v>
+        <v>+1h21min</v>
       </c>
       <c r="D50">
-        <v>-179</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B51" t="str">
-        <v>Eduarda Pereira Costa Silva</v>
+        <v>Raquele Fragoso Da Silva</v>
       </c>
       <c r="C51" t="str">
-        <v>+0h37min</v>
+        <v>-35h27min</v>
       </c>
       <c r="D51">
-        <v>37</v>
+        <v>-2127</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B52" t="str">
-        <v>Gabrielle Vitoria dos Santos</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
       <c r="C52" t="str">
-        <v>-6h23min</v>
+        <v>-2h59min</v>
       </c>
       <c r="D52">
-        <v>-383</v>
+        <v>-179</v>
       </c>
     </row>
     <row r="53">
@@ -1138,13 +1132,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B53" t="str">
-        <v>Larissa Alexia da Silva Souza</v>
+        <v>Eduarda Pereira Costa Silva</v>
       </c>
       <c r="C53" t="str">
-        <v>-3h32min</v>
+        <v>+0h37min</v>
       </c>
       <c r="D53">
-        <v>-212</v>
+        <v>37</v>
       </c>
     </row>
     <row r="54">
@@ -1152,13 +1146,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B54" t="str">
-        <v>Maria Cicília Brito Veiga</v>
+        <v>Larissa Alexia da Silva Souza</v>
       </c>
       <c r="C54" t="str">
-        <v>-3h41min</v>
+        <v>-3h32min</v>
       </c>
       <c r="D54">
-        <v>-221</v>
+        <v>-212</v>
       </c>
     </row>
     <row r="55">
@@ -1166,13 +1160,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B55" t="str">
-        <v>Maryanna Francielly Trajano da Silva</v>
+        <v>Maria Cicília Brito Veiga</v>
       </c>
       <c r="C55" t="str">
-        <v>-18h50min</v>
+        <v>-3h41min</v>
       </c>
       <c r="D55">
-        <v>-1130</v>
+        <v>-221</v>
       </c>
     </row>
     <row r="56">
@@ -1180,13 +1174,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B56" t="str">
-        <v>Robéria Gilo Da Silva</v>
+        <v>Maryanna Francielly Trajano da Silva</v>
       </c>
       <c r="C56" t="str">
-        <v>+53h25min</v>
+        <v>-18h50min</v>
       </c>
       <c r="D56">
-        <v>3205</v>
+        <v>-1130</v>
       </c>
     </row>
     <row r="57">
@@ -1197,10 +1191,10 @@
         <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
       <c r="C57" t="str">
-        <v>+19h52min</v>
+        <v>+19h32min</v>
       </c>
       <c r="D57">
-        <v>1192</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="58">
@@ -1222,41 +1216,41 @@
         <v>Leidiane Souza</v>
       </c>
       <c r="B59" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="C59" t="str">
-        <v>-19h5min</v>
+        <v>+0h</v>
       </c>
       <c r="D59">
-        <v>-1145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
+        <v>Leidiane Souza</v>
+      </c>
+      <c r="B60" t="str">
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
-      <c r="B60" t="str">
-        <v>Ana Paula Amaral Santos Ismerim</v>
-      </c>
       <c r="C60" t="str">
-        <v>-28h34min</v>
+        <v>+0h</v>
       </c>
       <c r="D60">
-        <v>-1714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="B61" t="str">
-        <v>Bruna Rayane Oliveira dos Santos</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="C61" t="str">
-        <v>+7h13min</v>
+        <v>-18h2min</v>
       </c>
       <c r="D61">
-        <v>433</v>
+        <v>-1082</v>
       </c>
     </row>
     <row r="62">
@@ -1264,13 +1258,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B62" t="str">
-        <v>Camille Kauane Da Silva Nunes</v>
+        <v>Ana Paula Amaral Santos Ismerim</v>
       </c>
       <c r="C62" t="str">
-        <v>+4h59min</v>
+        <v>-28h34min</v>
       </c>
       <c r="D62">
-        <v>299</v>
+        <v>-1714</v>
       </c>
     </row>
     <row r="63">
@@ -1278,13 +1272,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B63" t="str">
-        <v>Cristielle Pereira Lima Da Silva</v>
+        <v>Bruna Rayane Oliveira dos Santos</v>
       </c>
       <c r="C63" t="str">
-        <v>-18h14min</v>
+        <v>+7h13min</v>
       </c>
       <c r="D63">
-        <v>-1094</v>
+        <v>433</v>
       </c>
     </row>
     <row r="64">
@@ -1292,13 +1286,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B64" t="str">
-        <v>Deise Gislaine Silva vitor</v>
+        <v>Camille Kauane Da Silva Nunes</v>
       </c>
       <c r="C64" t="str">
-        <v>+22h59min</v>
+        <v>+6h23min</v>
       </c>
       <c r="D64">
-        <v>1379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="65">
@@ -1306,13 +1300,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B65" t="str">
-        <v>Eliene Da Silva Santos</v>
+        <v>Cristielle Pereira Lima Da Silva</v>
       </c>
       <c r="C65" t="str">
-        <v>+85h10min</v>
+        <v>-18h14min</v>
       </c>
       <c r="D65">
-        <v>5110</v>
+        <v>-1094</v>
       </c>
     </row>
     <row r="66">
@@ -1320,13 +1314,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B66" t="str">
-        <v>Maria Tatiane Basto Cardoso</v>
+        <v>Deise Gislaine Silva vitor</v>
       </c>
       <c r="C66" t="str">
-        <v>+56h4min</v>
+        <v>+22h59min</v>
       </c>
       <c r="D66">
-        <v>3364</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="67">
@@ -1334,13 +1328,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B67" t="str">
-        <v>Samyra Anchieta Bispo</v>
+        <v>Eliene Da Silva Santos</v>
       </c>
       <c r="C67" t="str">
-        <v>-2h32min</v>
+        <v>+85h10min</v>
       </c>
       <c r="D67">
-        <v>-152</v>
+        <v>5110</v>
       </c>
     </row>
     <row r="68">
@@ -1348,41 +1342,41 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B68" t="str">
-        <v>THAMIRYS SILVESTRINI MORALES</v>
+        <v>Maria Tatiane Basto Cardoso</v>
       </c>
       <c r="C68" t="str">
-        <v>-6h7min</v>
+        <v>+56h4min</v>
       </c>
       <c r="D68">
-        <v>-367</v>
+        <v>3364</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B69" t="str">
-        <v>Amanda Santos Costa</v>
+        <v>Samyra Anchieta Bispo</v>
       </c>
       <c r="C69" t="str">
-        <v>-37h20min</v>
+        <v>-2h32min</v>
       </c>
       <c r="D69">
-        <v>-2240</v>
+        <v>-152</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B70" t="str">
-        <v>Josimara Ferreira Monteiro</v>
+        <v>THAMIRYS SILVESTRINI MORALES</v>
       </c>
       <c r="C70" t="str">
-        <v>-19h23min</v>
+        <v>-6h7min</v>
       </c>
       <c r="D70">
-        <v>-1163</v>
+        <v>-367</v>
       </c>
     </row>
     <row r="71">
@@ -1390,13 +1384,13 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B71" t="str">
-        <v>Juliene bezerra</v>
+        <v>Amanda Santos Costa</v>
       </c>
       <c r="C71" t="str">
-        <v>-31h57min</v>
+        <v>-37h20min</v>
       </c>
       <c r="D71">
-        <v>-1917</v>
+        <v>-2240</v>
       </c>
     </row>
     <row r="72">
@@ -1404,13 +1398,13 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B72" t="str">
-        <v>Luís Henrique Batista dos Santos</v>
+        <v>Josimara Ferreira Monteiro</v>
       </c>
       <c r="C72" t="str">
-        <v>+0h</v>
+        <v>-19h23min</v>
       </c>
       <c r="D72">
-        <v>0</v>
+        <v>-1163</v>
       </c>
     </row>
     <row r="73">
@@ -1418,13 +1412,13 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B73" t="str">
-        <v>Maria Nobre Farias De França</v>
+        <v>Juliene bezerra</v>
       </c>
       <c r="C73" t="str">
-        <v>-36h1min</v>
+        <v>-31h57min</v>
       </c>
       <c r="D73">
-        <v>-2161</v>
+        <v>-1917</v>
       </c>
     </row>
     <row r="74">
@@ -1432,69 +1426,69 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B74" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Luís Henrique Batista dos Santos</v>
       </c>
       <c r="C74" t="str">
-        <v>-56h46min</v>
+        <v>+0h</v>
       </c>
       <c r="D74">
-        <v>-3406</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Rafaela Alves Mendes</v>
+        <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B75" t="str">
-        <v>Letícia Soares Belo</v>
+        <v>Maria Nobre Farias De França</v>
       </c>
       <c r="C75" t="str">
-        <v>-30h30min</v>
+        <v>+104h38min</v>
       </c>
       <c r="D75">
-        <v>-1830</v>
+        <v>6278</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Rafaela Alves Mendes</v>
+        <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B76" t="str">
-        <v>Millena Sthefany dos Santos Cruz</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="C76" t="str">
-        <v>+0h</v>
+        <v>-56h46min</v>
       </c>
       <c r="D76">
-        <v>0</v>
+        <v>-3406</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Rafaela Alves Mendes</v>
       </c>
       <c r="B77" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Letícia Soares Belo</v>
       </c>
       <c r="C77" t="str">
-        <v>+29h36min</v>
+        <v>-30h30min</v>
       </c>
       <c r="D77">
-        <v>1776</v>
+        <v>-1830</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Rafaela Alves Mendes</v>
       </c>
       <c r="B78" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Millena Sthefany dos Santos Cruz</v>
       </c>
       <c r="C78" t="str">
-        <v>-32h2min</v>
+        <v>+0h</v>
       </c>
       <c r="D78">
-        <v>-1922</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -1502,13 +1496,13 @@
         <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B79" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="C79" t="str">
-        <v>-29h22min</v>
+        <v>+29h36min</v>
       </c>
       <c r="D79">
-        <v>-1762</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="80">
@@ -1516,41 +1510,41 @@
         <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B80" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="C80" t="str">
-        <v>-21h14min</v>
+        <v>-32h2min</v>
       </c>
       <c r="D80">
-        <v>-1274</v>
+        <v>-1922</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Sem Gestor</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B81" t="str">
-        <v>Alberto Guilherme Da Silva Martins</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="C81" t="str">
-        <v>-27h11min</v>
+        <v>-29h22min</v>
       </c>
       <c r="D81">
-        <v>-1631</v>
+        <v>-1762</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Sem Gestor</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B82" t="str">
-        <v>Brunna Isabelly Silva lima</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="C82" t="str">
-        <v>-8h</v>
+        <v>-21h14min</v>
       </c>
       <c r="D82">
-        <v>-480</v>
+        <v>-1274</v>
       </c>
     </row>
     <row r="83">
@@ -1558,13 +1552,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B83" t="str">
-        <v>CLÉDJON DIAS DOS SANTOS</v>
+        <v>Alberto Guilherme Da Silva Martins</v>
       </c>
       <c r="C83" t="str">
-        <v>-522h28min</v>
+        <v>-27h11min</v>
       </c>
       <c r="D83">
-        <v>-31348</v>
+        <v>-1631</v>
       </c>
     </row>
     <row r="84">
@@ -1572,13 +1566,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B84" t="str">
-        <v>Leidiane Souza</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="C84" t="str">
-        <v>-4896h</v>
+        <v>+0h</v>
       </c>
       <c r="D84">
-        <v>-293760</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1586,13 +1580,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B85" t="str">
-        <v>Luiz Henrique Martins Tavares</v>
+        <v>Brunna Isabelly Silva lima</v>
       </c>
       <c r="C85" t="str">
-        <v>-4896h</v>
+        <v>-8h</v>
       </c>
       <c r="D85">
-        <v>-293760</v>
+        <v>-480</v>
       </c>
     </row>
     <row r="86">
@@ -1600,13 +1594,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B86" t="str">
-        <v>Maria Jeane da Silva Santos</v>
+        <v>CLÉDJON DIAS DOS SANTOS</v>
       </c>
       <c r="C86" t="str">
-        <v>+2h59min</v>
+        <v>-522h28min</v>
       </c>
       <c r="D86">
-        <v>179</v>
+        <v>-31348</v>
       </c>
     </row>
     <row r="87">
@@ -1614,13 +1608,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B87" t="str">
-        <v>Moises Santiago</v>
+        <v>Joanna Roberta de Queiroz Viana</v>
       </c>
       <c r="C87" t="str">
-        <v>-3148h</v>
+        <v>+0h</v>
       </c>
       <c r="D87">
-        <v>-188880</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -1628,7 +1622,7 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B88" t="str">
-        <v>Paulo Rogério Santos</v>
+        <v>José Fernando Dos Santos Santana Ramos</v>
       </c>
       <c r="C88" t="str">
         <v>+0h</v>
@@ -1639,63 +1633,189 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B89" t="str">
-        <v>João Ricardo Dantas Albuquerque</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="C89" t="str">
-        <v>-18h58min</v>
+        <v>-4896h</v>
       </c>
       <c r="D89">
-        <v>-1138</v>
+        <v>-293760</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B90" t="str">
-        <v>Lianda Melinda Santos Calixto</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="C90" t="str">
-        <v>-23h48min</v>
+        <v>+0h</v>
       </c>
       <c r="D90">
-        <v>-1428</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B91" t="str">
-        <v>Ravy Thiago Vieira Da Silva</v>
+        <v>Luiz Henrique Martins Tavares</v>
       </c>
       <c r="C91" t="str">
-        <v>+27h35min</v>
+        <v>-4896h</v>
       </c>
       <c r="D91">
-        <v>1655</v>
+        <v>-293760</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
+        <v>Sem Gestor</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Michaell Jean Nunes De Carvalho</v>
+      </c>
+      <c r="C92" t="str">
+        <v>+0h</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Sem Gestor</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Moises Santiago</v>
+      </c>
+      <c r="C93" t="str">
+        <v>-3148h</v>
+      </c>
+      <c r="D93">
+        <v>-188880</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Sem Gestor</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Paulo Rogério Santos</v>
+      </c>
+      <c r="C94" t="str">
+        <v>+0h</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Sem Gestor</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Rafaela Alves Mendes</v>
+      </c>
+      <c r="C95" t="str">
+        <v>+0h</v>
+      </c>
+      <c r="D95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Sem Gestor</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Romulo Jose Santos Lisboa</v>
+      </c>
+      <c r="C96" t="str">
+        <v>+0h</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Sem Gestor</v>
+      </c>
+      <c r="B97" t="str">
         <v>Suzana Martins Tavares</v>
       </c>
-      <c r="B92" t="str">
+      <c r="C97" t="str">
+        <v>+0h</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B98" t="str">
+        <v>João Ricardo Dantas Albuquerque</v>
+      </c>
+      <c r="C98" t="str">
+        <v>-18h58min</v>
+      </c>
+      <c r="D98">
+        <v>-1138</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Lianda Melinda Santos Calixto</v>
+      </c>
+      <c r="C99" t="str">
+        <v>-23h48min</v>
+      </c>
+      <c r="D99">
+        <v>-1428</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Ravy Thiago Vieira Da Silva</v>
+      </c>
+      <c r="C100" t="str">
+        <v>+27h35min</v>
+      </c>
+      <c r="D100">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B101" t="str">
         <v>Thayane Mayara dos Santos</v>
       </c>
-      <c r="C92" t="str">
+      <c r="C101" t="str">
         <v>-64h4min</v>
       </c>
-      <c r="D92">
+      <c r="D101">
         <v>-3844</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dados - 09/04/2026  8:34
</commit_message>
<xml_diff>
--- a/public/saldo_por_gestor.xlsx
+++ b/public/saldo_por_gestor.xlsx
@@ -397,7 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D92"/>
+  <cols>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,10 +455,10 @@
         <v>Claudio Bispo Dos Santos</v>
       </c>
       <c r="C4" t="str">
-        <v>-114h46min</v>
+        <v>-14h22min</v>
       </c>
       <c r="D4">
-        <v>-6886</v>
+        <v>-862</v>
       </c>
     </row>
     <row r="5">
@@ -561,10 +567,10 @@
         <v>Paulo Cesar Da Silva Santos Junior</v>
       </c>
       <c r="C12" t="str">
-        <v>-52h48min</v>
+        <v>-27h</v>
       </c>
       <c r="D12">
-        <v>-3168</v>
+        <v>-1620</v>
       </c>
     </row>
     <row r="13">
@@ -586,13 +592,13 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B14" t="str">
-        <v>Robéria Gilo Da Silva</v>
+        <v>Rosilene Martins Da Silva</v>
       </c>
       <c r="C14" t="str">
-        <v>-47h35min</v>
+        <v>-35h16min</v>
       </c>
       <c r="D14">
-        <v>-2855</v>
+        <v>-2116</v>
       </c>
     </row>
     <row r="15">
@@ -600,13 +606,13 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B15" t="str">
-        <v>Rosilene Martins Da Silva</v>
+        <v>Thalys Gomes Dos Santos</v>
       </c>
       <c r="C15" t="str">
-        <v>-35h16min</v>
+        <v>-42h4min</v>
       </c>
       <c r="D15">
-        <v>-2116</v>
+        <v>-2524</v>
       </c>
     </row>
     <row r="16">
@@ -614,27 +620,27 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B16" t="str">
-        <v>Thalys Gomes Dos Santos</v>
+        <v>Yuri Castro Gomes</v>
       </c>
       <c r="C16" t="str">
-        <v>-42h4min</v>
+        <v>+30h18min</v>
       </c>
       <c r="D16">
-        <v>-2524</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B17" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Ane Caroline Pereira marter</v>
       </c>
       <c r="C17" t="str">
-        <v>+30h18min</v>
+        <v>+11h23min</v>
       </c>
       <c r="D17">
-        <v>1818</v>
+        <v>683</v>
       </c>
     </row>
     <row r="18">
@@ -642,13 +648,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B18" t="str">
-        <v>Ane Caroline Pereira marter</v>
+        <v>Anny Karoline Andrade Santos</v>
       </c>
       <c r="C18" t="str">
-        <v>+11h23min</v>
+        <v>-44h19min</v>
       </c>
       <c r="D18">
-        <v>683</v>
+        <v>-2659</v>
       </c>
     </row>
     <row r="19">
@@ -656,13 +662,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B19" t="str">
-        <v>Anny Karoline Andrade Santos</v>
+        <v>Kamilla Santos da Silva</v>
       </c>
       <c r="C19" t="str">
-        <v>-44h19min</v>
+        <v>-23h12min</v>
       </c>
       <c r="D19">
-        <v>-2659</v>
+        <v>-1392</v>
       </c>
     </row>
     <row r="20">
@@ -670,13 +676,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B20" t="str">
-        <v>Kamilla Santos da Silva</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
       <c r="C20" t="str">
-        <v>-23h12min</v>
+        <v>+20h3min</v>
       </c>
       <c r="D20">
-        <v>-1392</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="21">
@@ -684,13 +690,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B21" t="str">
-        <v>Maria Jeane da Silva Santos</v>
+        <v>Sandra da Conceição Freitas</v>
       </c>
       <c r="C21" t="str">
-        <v>+2h59min</v>
+        <v>+5h6min</v>
       </c>
       <c r="D21">
-        <v>179</v>
+        <v>306</v>
       </c>
     </row>
     <row r="22">
@@ -698,55 +704,55 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B22" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Thamires Emanuelle da Silva</v>
       </c>
       <c r="C22" t="str">
-        <v>+20h3min</v>
+        <v>-2h26min</v>
       </c>
       <c r="D22">
-        <v>1203</v>
+        <v>-146</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B23" t="str">
-        <v>Sandra da Conceição Freitas</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="C23" t="str">
-        <v>+5h6min</v>
+        <v>-61h48min</v>
       </c>
       <c r="D23">
-        <v>306</v>
+        <v>-3708</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B24" t="str">
-        <v>Thamires Emanuelle da Silva</v>
+        <v>Ana Luiza Dos Santos</v>
       </c>
       <c r="C24" t="str">
-        <v>-2h26min</v>
+        <v>-29h7min</v>
       </c>
       <c r="D24">
-        <v>-146</v>
+        <v>-1747</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B25" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Emanoelle Feitosa Vieira Santos</v>
       </c>
       <c r="C25" t="str">
-        <v>-61h48min</v>
+        <v>-31h57min</v>
       </c>
       <c r="D25">
-        <v>-3708</v>
+        <v>-1917</v>
       </c>
     </row>
     <row r="26">
@@ -754,13 +760,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B26" t="str">
-        <v>Ana Luiza Dos Santos</v>
+        <v>Gessica Aparecida Dos Santos</v>
       </c>
       <c r="C26" t="str">
-        <v>-76h31min</v>
+        <v>-96h27min</v>
       </c>
       <c r="D26">
-        <v>-4591</v>
+        <v>-5787</v>
       </c>
     </row>
     <row r="27">
@@ -768,13 +774,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B27" t="str">
-        <v>Emanoelle Feitosa Vieira Santos</v>
+        <v>Giselle Dos Santos Roberto</v>
       </c>
       <c r="C27" t="str">
-        <v>-31h57min</v>
+        <v>-47h7min</v>
       </c>
       <c r="D27">
-        <v>-1917</v>
+        <v>-2827</v>
       </c>
     </row>
     <row r="28">
@@ -782,13 +788,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B28" t="str">
-        <v>Gessica Aparecida Dos Santos</v>
+        <v>Kauanne Iwashita Da Silva</v>
       </c>
       <c r="C28" t="str">
-        <v>-122h57min</v>
+        <v>-32h13min</v>
       </c>
       <c r="D28">
-        <v>-7377</v>
+        <v>-1933</v>
       </c>
     </row>
     <row r="29">
@@ -796,13 +802,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B29" t="str">
-        <v>Giselle Dos Santos Roberto</v>
+        <v>Laís Manuelle Santos Pereira</v>
       </c>
       <c r="C29" t="str">
-        <v>-47h7min</v>
+        <v>-16h57min</v>
       </c>
       <c r="D29">
-        <v>-2827</v>
+        <v>-1017</v>
       </c>
     </row>
     <row r="30">
@@ -810,13 +816,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B30" t="str">
-        <v>Kauanne Iwashita Da Silva</v>
+        <v>Leticia Seixas Santos</v>
       </c>
       <c r="C30" t="str">
-        <v>-224h49min</v>
+        <v>-16h41min</v>
       </c>
       <c r="D30">
-        <v>-13489</v>
+        <v>-1001</v>
       </c>
     </row>
     <row r="31">
@@ -824,13 +830,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B31" t="str">
-        <v>Laís Manuelle Santos Pereira</v>
+        <v>Luciene Da Silva Nascimento</v>
       </c>
       <c r="C31" t="str">
-        <v>-16h57min</v>
+        <v>-39h36min</v>
       </c>
       <c r="D31">
-        <v>-1017</v>
+        <v>-2376</v>
       </c>
     </row>
     <row r="32">
@@ -838,13 +844,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B32" t="str">
-        <v>Leticia Seixas Santos</v>
+        <v>Natali de Souza Gonzaga</v>
       </c>
       <c r="C32" t="str">
-        <v>-12h19min</v>
+        <v>-58h39min</v>
       </c>
       <c r="D32">
-        <v>-739</v>
+        <v>-3519</v>
       </c>
     </row>
     <row r="33">
@@ -852,13 +858,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B33" t="str">
-        <v>Luciene Da Silva Nascimento</v>
+        <v>Nathalia Vieira Lima</v>
       </c>
       <c r="C33" t="str">
-        <v>-10h35min</v>
+        <v>-73h26min</v>
       </c>
       <c r="D33">
-        <v>-635</v>
+        <v>-4406</v>
       </c>
     </row>
     <row r="34">
@@ -866,41 +872,41 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B34" t="str">
-        <v>Natali de Souza Gonzaga</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
       <c r="C34" t="str">
-        <v>-58h39min</v>
+        <v>+0h</v>
       </c>
       <c r="D34">
-        <v>-3519</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B35" t="str">
-        <v>Nathalia Vieira Lima</v>
+        <v>Fabia Batista da Silva</v>
       </c>
       <c r="C35" t="str">
-        <v>-73h4min</v>
+        <v>-26h19min</v>
       </c>
       <c r="D35">
-        <v>-4384</v>
+        <v>-1579</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B36" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Gessyca Nayara Rocha Santos</v>
       </c>
       <c r="C36" t="str">
-        <v>-188h</v>
+        <v>-43h12min</v>
       </c>
       <c r="D36">
-        <v>-11280</v>
+        <v>-2592</v>
       </c>
     </row>
     <row r="37">
@@ -908,13 +914,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B37" t="str">
-        <v>Fabia Batista da Silva</v>
+        <v>Jaine Mariana Rodrigues Mendonça</v>
       </c>
       <c r="C37" t="str">
-        <v>-26h19min</v>
+        <v>-3h42min</v>
       </c>
       <c r="D37">
-        <v>-1579</v>
+        <v>-222</v>
       </c>
     </row>
     <row r="38">
@@ -922,13 +928,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B38" t="str">
-        <v>Gessyca Nayara Rocha Santos</v>
+        <v>Karine Celestino Evangelista dos Santos</v>
       </c>
       <c r="C38" t="str">
-        <v>-156h27min</v>
+        <v>-12h53min</v>
       </c>
       <c r="D38">
-        <v>-9387</v>
+        <v>-773</v>
       </c>
     </row>
     <row r="39">
@@ -936,41 +942,41 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B39" t="str">
-        <v>Jaine Mariana Rodrigues Mendonça</v>
+        <v>Maria Tatiane Oliveira Santos</v>
       </c>
       <c r="C39" t="str">
-        <v>-3h42min</v>
+        <v>-52h59min</v>
       </c>
       <c r="D39">
-        <v>-222</v>
+        <v>-3179</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B40" t="str">
-        <v>Karine Celestino Evangelista dos Santos</v>
+        <v>Bruna Candido de Lima</v>
       </c>
       <c r="C40" t="str">
-        <v>-12h53min</v>
+        <v>+3h37min</v>
       </c>
       <c r="D40">
-        <v>-773</v>
+        <v>217</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B41" t="str">
-        <v>Maria Tatiane Oliveira Santos</v>
+        <v>Camilla Emanuelle Lopes de Almeida</v>
       </c>
       <c r="C41" t="str">
-        <v>-65h47min</v>
+        <v>-9h21min</v>
       </c>
       <c r="D41">
-        <v>-3947</v>
+        <v>-561</v>
       </c>
     </row>
     <row r="42">
@@ -978,13 +984,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B42" t="str">
-        <v>Bruna Candido de Lima</v>
+        <v>Danielle Dos Santos Silva</v>
       </c>
       <c r="C42" t="str">
-        <v>+3h37min</v>
+        <v>-26h55min</v>
       </c>
       <c r="D42">
-        <v>217</v>
+        <v>-1615</v>
       </c>
     </row>
     <row r="43">
@@ -992,13 +998,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B43" t="str">
-        <v>Camilla Emanuelle Lopes de Almeida</v>
+        <v>Edna Lopes Da Silva</v>
       </c>
       <c r="C43" t="str">
-        <v>-9h21min</v>
+        <v>+12h</v>
       </c>
       <c r="D43">
-        <v>-561</v>
+        <v>720</v>
       </c>
     </row>
     <row r="44">
@@ -1006,13 +1012,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B44" t="str">
-        <v>Danielle Dos Santos Silva</v>
+        <v>Jordelle Meygre Costa De Oliveira</v>
       </c>
       <c r="C44" t="str">
-        <v>-0h43min</v>
+        <v>+25h47min</v>
       </c>
       <c r="D44">
-        <v>-43</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="45">
@@ -1020,13 +1026,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B45" t="str">
-        <v>Edna Lopes Da Silva</v>
+        <v>Lays da Silva Vieira</v>
       </c>
       <c r="C45" t="str">
-        <v>+173h46min</v>
+        <v>+0h27min</v>
       </c>
       <c r="D45">
-        <v>10426</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46">
@@ -1034,13 +1040,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B46" t="str">
-        <v>Jordelle Meygre Costa De Oliveira</v>
+        <v>Luan Santos de Oliveira</v>
       </c>
       <c r="C46" t="str">
-        <v>+51h49min</v>
+        <v>+9h26min</v>
       </c>
       <c r="D46">
-        <v>3109</v>
+        <v>566</v>
       </c>
     </row>
     <row r="47">
@@ -1048,13 +1054,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B47" t="str">
-        <v>Lays da Silva Vieira</v>
+        <v>Maria Victoria Souza Araujo Ferro</v>
       </c>
       <c r="C47" t="str">
-        <v>+0h27min</v>
+        <v>-29h32min</v>
       </c>
       <c r="D47">
-        <v>27</v>
+        <v>-1772</v>
       </c>
     </row>
     <row r="48">
@@ -1062,13 +1068,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B48" t="str">
-        <v>Luan Santos de Oliveira</v>
+        <v>Marília Alice dos Santos Silva</v>
       </c>
       <c r="C48" t="str">
-        <v>+9h26min</v>
+        <v>+1h21min</v>
       </c>
       <c r="D48">
-        <v>566</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49">
@@ -1076,13 +1082,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B49" t="str">
-        <v>Maria Victoria Souza Araujo Ferro</v>
+        <v>Raquele Fragoso Da Silva</v>
       </c>
       <c r="C49" t="str">
-        <v>-29h32min</v>
+        <v>-35h27min</v>
       </c>
       <c r="D49">
-        <v>-1772</v>
+        <v>-2127</v>
       </c>
     </row>
     <row r="50">
@@ -1090,41 +1096,41 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B50" t="str">
-        <v>Marília Alice dos Santos Silva</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
       <c r="C50" t="str">
-        <v>+1h21min</v>
+        <v>-2h59min</v>
       </c>
       <c r="D50">
-        <v>81</v>
+        <v>-179</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B51" t="str">
-        <v>Raquele Fragoso Da Silva</v>
+        <v>Eduarda Pereira Costa Silva</v>
       </c>
       <c r="C51" t="str">
-        <v>-35h27min</v>
+        <v>+0h37min</v>
       </c>
       <c r="D51">
-        <v>-2127</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B52" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Gabrielle Vitoria dos Santos</v>
       </c>
       <c r="C52" t="str">
-        <v>-2h59min</v>
+        <v>-6h23min</v>
       </c>
       <c r="D52">
-        <v>-179</v>
+        <v>-383</v>
       </c>
     </row>
     <row r="53">
@@ -1132,13 +1138,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B53" t="str">
-        <v>Eduarda Pereira Costa Silva</v>
+        <v>Larissa Alexia da Silva Souza</v>
       </c>
       <c r="C53" t="str">
-        <v>+0h37min</v>
+        <v>-3h32min</v>
       </c>
       <c r="D53">
-        <v>37</v>
+        <v>-212</v>
       </c>
     </row>
     <row r="54">
@@ -1146,13 +1152,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B54" t="str">
-        <v>Larissa Alexia da Silva Souza</v>
+        <v>Maria Cicília Brito Veiga</v>
       </c>
       <c r="C54" t="str">
-        <v>-3h32min</v>
+        <v>-3h41min</v>
       </c>
       <c r="D54">
-        <v>-212</v>
+        <v>-221</v>
       </c>
     </row>
     <row r="55">
@@ -1160,13 +1166,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B55" t="str">
-        <v>Maria Cicília Brito Veiga</v>
+        <v>Maryanna Francielly Trajano da Silva</v>
       </c>
       <c r="C55" t="str">
-        <v>-3h41min</v>
+        <v>-18h50min</v>
       </c>
       <c r="D55">
-        <v>-221</v>
+        <v>-1130</v>
       </c>
     </row>
     <row r="56">
@@ -1174,13 +1180,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B56" t="str">
-        <v>Maryanna Francielly Trajano da Silva</v>
+        <v>Robéria Gilo Da Silva</v>
       </c>
       <c r="C56" t="str">
-        <v>-18h50min</v>
+        <v>+53h25min</v>
       </c>
       <c r="D56">
-        <v>-1130</v>
+        <v>3205</v>
       </c>
     </row>
     <row r="57">
@@ -1191,10 +1197,10 @@
         <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
       <c r="C57" t="str">
-        <v>+19h32min</v>
+        <v>+19h52min</v>
       </c>
       <c r="D57">
-        <v>1172</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="58">
@@ -1216,41 +1222,41 @@
         <v>Leidiane Souza</v>
       </c>
       <c r="B59" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="C59" t="str">
-        <v>+0h</v>
+        <v>-19h5min</v>
       </c>
       <c r="D59">
-        <v>0</v>
+        <v>-1145</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Leidiane Souza</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B60" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Ana Paula Amaral Santos Ismerim</v>
       </c>
       <c r="C60" t="str">
-        <v>+0h</v>
+        <v>-28h34min</v>
       </c>
       <c r="D60">
-        <v>0</v>
+        <v>-1714</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Leidiane Souza</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B61" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Bruna Rayane Oliveira dos Santos</v>
       </c>
       <c r="C61" t="str">
-        <v>-18h2min</v>
+        <v>+7h13min</v>
       </c>
       <c r="D61">
-        <v>-1082</v>
+        <v>433</v>
       </c>
     </row>
     <row r="62">
@@ -1258,13 +1264,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B62" t="str">
-        <v>Ana Paula Amaral Santos Ismerim</v>
+        <v>Camille Kauane Da Silva Nunes</v>
       </c>
       <c r="C62" t="str">
-        <v>-28h34min</v>
+        <v>+4h59min</v>
       </c>
       <c r="D62">
-        <v>-1714</v>
+        <v>299</v>
       </c>
     </row>
     <row r="63">
@@ -1272,13 +1278,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B63" t="str">
-        <v>Bruna Rayane Oliveira dos Santos</v>
+        <v>Cristielle Pereira Lima Da Silva</v>
       </c>
       <c r="C63" t="str">
-        <v>+7h13min</v>
+        <v>-18h14min</v>
       </c>
       <c r="D63">
-        <v>433</v>
+        <v>-1094</v>
       </c>
     </row>
     <row r="64">
@@ -1286,13 +1292,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B64" t="str">
-        <v>Camille Kauane Da Silva Nunes</v>
+        <v>Deise Gislaine Silva vitor</v>
       </c>
       <c r="C64" t="str">
-        <v>+6h23min</v>
+        <v>+22h59min</v>
       </c>
       <c r="D64">
-        <v>383</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="65">
@@ -1300,13 +1306,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B65" t="str">
-        <v>Cristielle Pereira Lima Da Silva</v>
+        <v>Eliene Da Silva Santos</v>
       </c>
       <c r="C65" t="str">
-        <v>-18h14min</v>
+        <v>+85h10min</v>
       </c>
       <c r="D65">
-        <v>-1094</v>
+        <v>5110</v>
       </c>
     </row>
     <row r="66">
@@ -1314,13 +1320,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B66" t="str">
-        <v>Deise Gislaine Silva vitor</v>
+        <v>Maria Tatiane Basto Cardoso</v>
       </c>
       <c r="C66" t="str">
-        <v>+22h59min</v>
+        <v>+56h4min</v>
       </c>
       <c r="D66">
-        <v>1379</v>
+        <v>3364</v>
       </c>
     </row>
     <row r="67">
@@ -1328,13 +1334,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B67" t="str">
-        <v>Eliene Da Silva Santos</v>
+        <v>Samyra Anchieta Bispo</v>
       </c>
       <c r="C67" t="str">
-        <v>+85h10min</v>
+        <v>-2h32min</v>
       </c>
       <c r="D67">
-        <v>5110</v>
+        <v>-152</v>
       </c>
     </row>
     <row r="68">
@@ -1342,41 +1348,41 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B68" t="str">
-        <v>Maria Tatiane Basto Cardoso</v>
+        <v>THAMIRYS SILVESTRINI MORALES</v>
       </c>
       <c r="C68" t="str">
-        <v>+56h4min</v>
+        <v>-6h7min</v>
       </c>
       <c r="D68">
-        <v>3364</v>
+        <v>-367</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B69" t="str">
-        <v>Samyra Anchieta Bispo</v>
+        <v>Amanda Santos Costa</v>
       </c>
       <c r="C69" t="str">
-        <v>-2h32min</v>
+        <v>-37h20min</v>
       </c>
       <c r="D69">
-        <v>-152</v>
+        <v>-2240</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B70" t="str">
-        <v>THAMIRYS SILVESTRINI MORALES</v>
+        <v>Josimara Ferreira Monteiro</v>
       </c>
       <c r="C70" t="str">
-        <v>-6h7min</v>
+        <v>-19h23min</v>
       </c>
       <c r="D70">
-        <v>-367</v>
+        <v>-1163</v>
       </c>
     </row>
     <row r="71">
@@ -1384,13 +1390,13 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B71" t="str">
-        <v>Amanda Santos Costa</v>
+        <v>Juliene bezerra</v>
       </c>
       <c r="C71" t="str">
-        <v>-37h20min</v>
+        <v>-31h57min</v>
       </c>
       <c r="D71">
-        <v>-2240</v>
+        <v>-1917</v>
       </c>
     </row>
     <row r="72">
@@ -1398,13 +1404,13 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B72" t="str">
-        <v>Josimara Ferreira Monteiro</v>
+        <v>Luís Henrique Batista dos Santos</v>
       </c>
       <c r="C72" t="str">
-        <v>-19h23min</v>
+        <v>+0h</v>
       </c>
       <c r="D72">
-        <v>-1163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1412,13 +1418,13 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B73" t="str">
-        <v>Juliene bezerra</v>
+        <v>Maria Nobre Farias De França</v>
       </c>
       <c r="C73" t="str">
-        <v>-31h57min</v>
+        <v>-36h1min</v>
       </c>
       <c r="D73">
-        <v>-1917</v>
+        <v>-2161</v>
       </c>
     </row>
     <row r="74">
@@ -1426,69 +1432,69 @@
         <v>Michaell Jean Nunes De Carvalho</v>
       </c>
       <c r="B74" t="str">
-        <v>Luís Henrique Batista dos Santos</v>
+        <v>Tomás Azevedo Santos</v>
       </c>
       <c r="C74" t="str">
-        <v>+0h</v>
+        <v>-56h46min</v>
       </c>
       <c r="D74">
-        <v>0</v>
+        <v>-3406</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Rafaela Alves Mendes</v>
       </c>
       <c r="B75" t="str">
-        <v>Maria Nobre Farias De França</v>
+        <v>Letícia Soares Belo</v>
       </c>
       <c r="C75" t="str">
-        <v>+104h38min</v>
+        <v>-30h30min</v>
       </c>
       <c r="D75">
-        <v>6278</v>
+        <v>-1830</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Rafaela Alves Mendes</v>
       </c>
       <c r="B76" t="str">
-        <v>Tomás Azevedo Santos</v>
+        <v>Millena Sthefany dos Santos Cruz</v>
       </c>
       <c r="C76" t="str">
-        <v>-56h46min</v>
+        <v>+0h</v>
       </c>
       <c r="D76">
-        <v>-3406</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Rafaela Alves Mendes</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B77" t="str">
-        <v>Letícia Soares Belo</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="C77" t="str">
-        <v>-30h30min</v>
+        <v>+29h36min</v>
       </c>
       <c r="D77">
-        <v>-1830</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Rafaela Alves Mendes</v>
+        <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B78" t="str">
-        <v>Millena Sthefany dos Santos Cruz</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="C78" t="str">
-        <v>+0h</v>
+        <v>-32h2min</v>
       </c>
       <c r="D78">
-        <v>0</v>
+        <v>-1922</v>
       </c>
     </row>
     <row r="79">
@@ -1496,13 +1502,13 @@
         <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B79" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="C79" t="str">
-        <v>+29h36min</v>
+        <v>-29h22min</v>
       </c>
       <c r="D79">
-        <v>1776</v>
+        <v>-1762</v>
       </c>
     </row>
     <row r="80">
@@ -1510,41 +1516,41 @@
         <v>Romulo Jose Santos Lisboa</v>
       </c>
       <c r="B80" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="C80" t="str">
-        <v>-32h2min</v>
+        <v>-21h14min</v>
       </c>
       <c r="D80">
-        <v>-1922</v>
+        <v>-1274</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B81" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Alberto Guilherme Da Silva Martins</v>
       </c>
       <c r="C81" t="str">
-        <v>-29h22min</v>
+        <v>-27h11min</v>
       </c>
       <c r="D81">
-        <v>-1762</v>
+        <v>-1631</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B82" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Brunna Isabelly Silva lima</v>
       </c>
       <c r="C82" t="str">
-        <v>-21h14min</v>
+        <v>-8h</v>
       </c>
       <c r="D82">
-        <v>-1274</v>
+        <v>-480</v>
       </c>
     </row>
     <row r="83">
@@ -1552,13 +1558,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B83" t="str">
-        <v>Alberto Guilherme Da Silva Martins</v>
+        <v>CLÉDJON DIAS DOS SANTOS</v>
       </c>
       <c r="C83" t="str">
-        <v>-27h11min</v>
+        <v>-522h28min</v>
       </c>
       <c r="D83">
-        <v>-1631</v>
+        <v>-31348</v>
       </c>
     </row>
     <row r="84">
@@ -1566,13 +1572,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B84" t="str">
-        <v>Alberto Luiz Marinho Batista</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="C84" t="str">
-        <v>+0h</v>
+        <v>-4896h</v>
       </c>
       <c r="D84">
-        <v>0</v>
+        <v>-293760</v>
       </c>
     </row>
     <row r="85">
@@ -1580,13 +1586,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B85" t="str">
-        <v>Brunna Isabelly Silva lima</v>
+        <v>Luiz Henrique Martins Tavares</v>
       </c>
       <c r="C85" t="str">
-        <v>-8h</v>
+        <v>-4896h</v>
       </c>
       <c r="D85">
-        <v>-480</v>
+        <v>-293760</v>
       </c>
     </row>
     <row r="86">
@@ -1594,13 +1600,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B86" t="str">
-        <v>CLÉDJON DIAS DOS SANTOS</v>
+        <v>Maria Jeane da Silva Santos</v>
       </c>
       <c r="C86" t="str">
-        <v>-522h28min</v>
+        <v>+2h59min</v>
       </c>
       <c r="D86">
-        <v>-31348</v>
+        <v>179</v>
       </c>
     </row>
     <row r="87">
@@ -1608,13 +1614,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B87" t="str">
-        <v>Joanna Roberta de Queiroz Viana</v>
+        <v>Moises Santiago</v>
       </c>
       <c r="C87" t="str">
-        <v>+0h</v>
+        <v>-3148h</v>
       </c>
       <c r="D87">
-        <v>0</v>
+        <v>-188880</v>
       </c>
     </row>
     <row r="88">
@@ -1622,7 +1628,7 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B88" t="str">
-        <v>José Fernando Dos Santos Santana Ramos</v>
+        <v>Paulo Rogério Santos</v>
       </c>
       <c r="C88" t="str">
         <v>+0h</v>
@@ -1633,189 +1639,63 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Sem Gestor</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B89" t="str">
-        <v>Leidiane Souza</v>
+        <v>João Ricardo Dantas Albuquerque</v>
       </c>
       <c r="C89" t="str">
-        <v>-4896h</v>
+        <v>-18h58min</v>
       </c>
       <c r="D89">
-        <v>-293760</v>
+        <v>-1138</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Sem Gestor</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B90" t="str">
-        <v>Leidiane Souza</v>
+        <v>Lianda Melinda Santos Calixto</v>
       </c>
       <c r="C90" t="str">
-        <v>+0h</v>
+        <v>-23h48min</v>
       </c>
       <c r="D90">
-        <v>0</v>
+        <v>-1428</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Sem Gestor</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B91" t="str">
-        <v>Luiz Henrique Martins Tavares</v>
+        <v>Ravy Thiago Vieira Da Silva</v>
       </c>
       <c r="C91" t="str">
-        <v>-4896h</v>
+        <v>+27h35min</v>
       </c>
       <c r="D91">
-        <v>-293760</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Sem Gestor</v>
+        <v>Suzana Martins Tavares</v>
       </c>
       <c r="B92" t="str">
-        <v>Michaell Jean Nunes De Carvalho</v>
+        <v>Thayane Mayara dos Santos</v>
       </c>
       <c r="C92" t="str">
-        <v>+0h</v>
+        <v>-64h4min</v>
       </c>
       <c r="D92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="str">
-        <v>Sem Gestor</v>
-      </c>
-      <c r="B93" t="str">
-        <v>Moises Santiago</v>
-      </c>
-      <c r="C93" t="str">
-        <v>-3148h</v>
-      </c>
-      <c r="D93">
-        <v>-188880</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="str">
-        <v>Sem Gestor</v>
-      </c>
-      <c r="B94" t="str">
-        <v>Paulo Rogério Santos</v>
-      </c>
-      <c r="C94" t="str">
-        <v>+0h</v>
-      </c>
-      <c r="D94">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <v>Sem Gestor</v>
-      </c>
-      <c r="B95" t="str">
-        <v>Rafaela Alves Mendes</v>
-      </c>
-      <c r="C95" t="str">
-        <v>+0h</v>
-      </c>
-      <c r="D95">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="str">
-        <v>Sem Gestor</v>
-      </c>
-      <c r="B96" t="str">
-        <v>Romulo Jose Santos Lisboa</v>
-      </c>
-      <c r="C96" t="str">
-        <v>+0h</v>
-      </c>
-      <c r="D96">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>Sem Gestor</v>
-      </c>
-      <c r="B97" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="C97" t="str">
-        <v>+0h</v>
-      </c>
-      <c r="D97">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B98" t="str">
-        <v>João Ricardo Dantas Albuquerque</v>
-      </c>
-      <c r="C98" t="str">
-        <v>-18h58min</v>
-      </c>
-      <c r="D98">
-        <v>-1138</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B99" t="str">
-        <v>Lianda Melinda Santos Calixto</v>
-      </c>
-      <c r="C99" t="str">
-        <v>-23h48min</v>
-      </c>
-      <c r="D99">
-        <v>-1428</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B100" t="str">
-        <v>Ravy Thiago Vieira Da Silva</v>
-      </c>
-      <c r="C100" t="str">
-        <v>+27h35min</v>
-      </c>
-      <c r="D100">
-        <v>1655</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>Suzana Martins Tavares</v>
-      </c>
-      <c r="B101" t="str">
-        <v>Thayane Mayara dos Santos</v>
-      </c>
-      <c r="C101" t="str">
-        <v>-64h4min</v>
-      </c>
-      <c r="D101">
         <v>-3844</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D92"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dados - 09/04/2026  8:42
</commit_message>
<xml_diff>
--- a/public/saldo_por_gestor.xlsx
+++ b/public/saldo_por_gestor.xlsx
@@ -398,12 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D92"/>
-  <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -455,10 +449,10 @@
         <v>Claudio Bispo Dos Santos</v>
       </c>
       <c r="C4" t="str">
-        <v>-14h22min</v>
+        <v>-12h50min</v>
       </c>
       <c r="D4">
-        <v>-862</v>
+        <v>-770</v>
       </c>
     </row>
     <row r="5">
@@ -592,13 +586,13 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B14" t="str">
-        <v>Rosilene Martins Da Silva</v>
+        <v>Robéria Gilo Da Silva</v>
       </c>
       <c r="C14" t="str">
-        <v>-35h16min</v>
+        <v>+53h25min</v>
       </c>
       <c r="D14">
-        <v>-2116</v>
+        <v>3205</v>
       </c>
     </row>
     <row r="15">
@@ -606,13 +600,13 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B15" t="str">
-        <v>Thalys Gomes Dos Santos</v>
+        <v>Rosilene Martins Da Silva</v>
       </c>
       <c r="C15" t="str">
-        <v>-42h4min</v>
+        <v>-35h16min</v>
       </c>
       <c r="D15">
-        <v>-2524</v>
+        <v>-2116</v>
       </c>
     </row>
     <row r="16">
@@ -620,27 +614,27 @@
         <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B16" t="str">
-        <v>Yuri Castro Gomes</v>
+        <v>Thalys Gomes Dos Santos</v>
       </c>
       <c r="C16" t="str">
-        <v>+30h18min</v>
+        <v>-42h4min</v>
       </c>
       <c r="D16">
-        <v>1818</v>
+        <v>-2524</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Alberto Luiz Marinho Batista</v>
       </c>
       <c r="B17" t="str">
-        <v>Ane Caroline Pereira marter</v>
+        <v>Yuri Castro Gomes</v>
       </c>
       <c r="C17" t="str">
-        <v>+11h23min</v>
+        <v>+30h18min</v>
       </c>
       <c r="D17">
-        <v>683</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="18">
@@ -648,13 +642,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B18" t="str">
-        <v>Anny Karoline Andrade Santos</v>
+        <v>Ane Caroline Pereira marter</v>
       </c>
       <c r="C18" t="str">
-        <v>-44h19min</v>
+        <v>+11h23min</v>
       </c>
       <c r="D18">
-        <v>-2659</v>
+        <v>683</v>
       </c>
     </row>
     <row r="19">
@@ -662,13 +656,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B19" t="str">
-        <v>Kamilla Santos da Silva</v>
+        <v>Anny Karoline Andrade Santos</v>
       </c>
       <c r="C19" t="str">
-        <v>-23h12min</v>
+        <v>-44h19min</v>
       </c>
       <c r="D19">
-        <v>-1392</v>
+        <v>-2659</v>
       </c>
     </row>
     <row r="20">
@@ -676,13 +670,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B20" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Kamilla Santos da Silva</v>
       </c>
       <c r="C20" t="str">
-        <v>+20h3min</v>
+        <v>-23h12min</v>
       </c>
       <c r="D20">
-        <v>1203</v>
+        <v>-1392</v>
       </c>
     </row>
     <row r="21">
@@ -690,13 +684,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B21" t="str">
-        <v>Sandra da Conceição Freitas</v>
+        <v>Maria Jeane da Silva Santos</v>
       </c>
       <c r="C21" t="str">
-        <v>+5h6min</v>
+        <v>+2h59min</v>
       </c>
       <c r="D21">
-        <v>306</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22">
@@ -704,55 +698,55 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B22" t="str">
-        <v>Thamires Emanuelle da Silva</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
       <c r="C22" t="str">
-        <v>-2h26min</v>
+        <v>+20h3min</v>
       </c>
       <c r="D22">
-        <v>-146</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B23" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Sandra da Conceição Freitas</v>
       </c>
       <c r="C23" t="str">
-        <v>-61h48min</v>
+        <v>+5h6min</v>
       </c>
       <c r="D23">
-        <v>-3708</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B24" t="str">
-        <v>Ana Luiza Dos Santos</v>
+        <v>Thamires Emanuelle da Silva</v>
       </c>
       <c r="C24" t="str">
-        <v>-29h7min</v>
+        <v>-2h26min</v>
       </c>
       <c r="D24">
-        <v>-1747</v>
+        <v>-146</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B25" t="str">
-        <v>Emanoelle Feitosa Vieira Santos</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="C25" t="str">
-        <v>-31h57min</v>
+        <v>-61h48min</v>
       </c>
       <c r="D25">
-        <v>-1917</v>
+        <v>-3708</v>
       </c>
     </row>
     <row r="26">
@@ -760,13 +754,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B26" t="str">
-        <v>Gessica Aparecida Dos Santos</v>
+        <v>Ana Luiza Dos Santos</v>
       </c>
       <c r="C26" t="str">
-        <v>-96h27min</v>
+        <v>-29h7min</v>
       </c>
       <c r="D26">
-        <v>-5787</v>
+        <v>-1747</v>
       </c>
     </row>
     <row r="27">
@@ -774,13 +768,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B27" t="str">
-        <v>Giselle Dos Santos Roberto</v>
+        <v>Emanoelle Feitosa Vieira Santos</v>
       </c>
       <c r="C27" t="str">
-        <v>-47h7min</v>
+        <v>-31h57min</v>
       </c>
       <c r="D27">
-        <v>-2827</v>
+        <v>-1917</v>
       </c>
     </row>
     <row r="28">
@@ -788,13 +782,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B28" t="str">
-        <v>Kauanne Iwashita Da Silva</v>
+        <v>Gessica Aparecida Dos Santos</v>
       </c>
       <c r="C28" t="str">
-        <v>-32h13min</v>
+        <v>-96h27min</v>
       </c>
       <c r="D28">
-        <v>-1933</v>
+        <v>-5787</v>
       </c>
     </row>
     <row r="29">
@@ -802,13 +796,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B29" t="str">
-        <v>Laís Manuelle Santos Pereira</v>
+        <v>Giselle Dos Santos Roberto</v>
       </c>
       <c r="C29" t="str">
-        <v>-16h57min</v>
+        <v>-47h7min</v>
       </c>
       <c r="D29">
-        <v>-1017</v>
+        <v>-2827</v>
       </c>
     </row>
     <row r="30">
@@ -816,13 +810,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B30" t="str">
-        <v>Leticia Seixas Santos</v>
+        <v>Kauanne Iwashita Da Silva</v>
       </c>
       <c r="C30" t="str">
-        <v>-16h41min</v>
+        <v>-32h13min</v>
       </c>
       <c r="D30">
-        <v>-1001</v>
+        <v>-1933</v>
       </c>
     </row>
     <row r="31">
@@ -830,13 +824,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B31" t="str">
-        <v>Luciene Da Silva Nascimento</v>
+        <v>Laís Manuelle Santos Pereira</v>
       </c>
       <c r="C31" t="str">
-        <v>-39h36min</v>
+        <v>-16h57min</v>
       </c>
       <c r="D31">
-        <v>-2376</v>
+        <v>-1017</v>
       </c>
     </row>
     <row r="32">
@@ -844,13 +838,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B32" t="str">
-        <v>Natali de Souza Gonzaga</v>
+        <v>Leticia Seixas Santos</v>
       </c>
       <c r="C32" t="str">
-        <v>-58h39min</v>
+        <v>-12h19min</v>
       </c>
       <c r="D32">
-        <v>-3519</v>
+        <v>-739</v>
       </c>
     </row>
     <row r="33">
@@ -858,13 +852,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B33" t="str">
-        <v>Nathalia Vieira Lima</v>
+        <v>Luciene Da Silva Nascimento</v>
       </c>
       <c r="C33" t="str">
-        <v>-73h26min</v>
+        <v>-39h36min</v>
       </c>
       <c r="D33">
-        <v>-4406</v>
+        <v>-2376</v>
       </c>
     </row>
     <row r="34">
@@ -872,41 +866,41 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B34" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Natali de Souza Gonzaga</v>
       </c>
       <c r="C34" t="str">
-        <v>+0h</v>
+        <v>-58h39min</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>-3519</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B35" t="str">
-        <v>Fabia Batista da Silva</v>
+        <v>Nathalia Vieira Lima</v>
       </c>
       <c r="C35" t="str">
-        <v>-26h19min</v>
+        <v>-73h26min</v>
       </c>
       <c r="D35">
-        <v>-1579</v>
+        <v>-4406</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B36" t="str">
-        <v>Gessyca Nayara Rocha Santos</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
       <c r="C36" t="str">
-        <v>-43h12min</v>
+        <v>+0h</v>
       </c>
       <c r="D36">
-        <v>-2592</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -914,13 +908,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B37" t="str">
-        <v>Jaine Mariana Rodrigues Mendonça</v>
+        <v>Fabia Batista da Silva</v>
       </c>
       <c r="C37" t="str">
-        <v>-3h42min</v>
+        <v>-26h19min</v>
       </c>
       <c r="D37">
-        <v>-222</v>
+        <v>-1579</v>
       </c>
     </row>
     <row r="38">
@@ -928,13 +922,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B38" t="str">
-        <v>Karine Celestino Evangelista dos Santos</v>
+        <v>Gessyca Nayara Rocha Santos</v>
       </c>
       <c r="C38" t="str">
-        <v>-12h53min</v>
+        <v>-43h12min</v>
       </c>
       <c r="D38">
-        <v>-773</v>
+        <v>-2592</v>
       </c>
     </row>
     <row r="39">
@@ -942,41 +936,41 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B39" t="str">
-        <v>Maria Tatiane Oliveira Santos</v>
+        <v>Jaine Mariana Rodrigues Mendonça</v>
       </c>
       <c r="C39" t="str">
-        <v>-52h59min</v>
+        <v>-3h42min</v>
       </c>
       <c r="D39">
-        <v>-3179</v>
+        <v>-222</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B40" t="str">
-        <v>Bruna Candido de Lima</v>
+        <v>Karine Celestino Evangelista dos Santos</v>
       </c>
       <c r="C40" t="str">
-        <v>+3h37min</v>
+        <v>-12h53min</v>
       </c>
       <c r="D40">
-        <v>217</v>
+        <v>-773</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B41" t="str">
-        <v>Camilla Emanuelle Lopes de Almeida</v>
+        <v>Maria Tatiane Oliveira Santos</v>
       </c>
       <c r="C41" t="str">
-        <v>-9h21min</v>
+        <v>-52h59min</v>
       </c>
       <c r="D41">
-        <v>-561</v>
+        <v>-3179</v>
       </c>
     </row>
     <row r="42">
@@ -984,13 +978,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B42" t="str">
-        <v>Danielle Dos Santos Silva</v>
+        <v>Bruna Candido de Lima</v>
       </c>
       <c r="C42" t="str">
-        <v>-26h55min</v>
+        <v>+3h37min</v>
       </c>
       <c r="D42">
-        <v>-1615</v>
+        <v>217</v>
       </c>
     </row>
     <row r="43">
@@ -998,13 +992,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B43" t="str">
-        <v>Edna Lopes Da Silva</v>
+        <v>Camilla Emanuelle Lopes de Almeida</v>
       </c>
       <c r="C43" t="str">
-        <v>+12h</v>
+        <v>-9h21min</v>
       </c>
       <c r="D43">
-        <v>720</v>
+        <v>-561</v>
       </c>
     </row>
     <row r="44">
@@ -1012,13 +1006,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B44" t="str">
-        <v>Jordelle Meygre Costa De Oliveira</v>
+        <v>Danielle Dos Santos Silva</v>
       </c>
       <c r="C44" t="str">
-        <v>+25h47min</v>
+        <v>-26h55min</v>
       </c>
       <c r="D44">
-        <v>1547</v>
+        <v>-1615</v>
       </c>
     </row>
     <row r="45">
@@ -1026,13 +1020,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B45" t="str">
-        <v>Lays da Silva Vieira</v>
+        <v>Edna Lopes Da Silva</v>
       </c>
       <c r="C45" t="str">
-        <v>+0h27min</v>
+        <v>+12h</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>720</v>
       </c>
     </row>
     <row r="46">
@@ -1040,13 +1034,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B46" t="str">
-        <v>Luan Santos de Oliveira</v>
+        <v>Jordelle Meygre Costa De Oliveira</v>
       </c>
       <c r="C46" t="str">
-        <v>+9h26min</v>
+        <v>+25h47min</v>
       </c>
       <c r="D46">
-        <v>566</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="47">
@@ -1054,13 +1048,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B47" t="str">
-        <v>Maria Victoria Souza Araujo Ferro</v>
+        <v>Lays da Silva Vieira</v>
       </c>
       <c r="C47" t="str">
-        <v>-29h32min</v>
+        <v>+0h27min</v>
       </c>
       <c r="D47">
-        <v>-1772</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48">
@@ -1068,13 +1062,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B48" t="str">
-        <v>Marília Alice dos Santos Silva</v>
+        <v>Luan Santos de Oliveira</v>
       </c>
       <c r="C48" t="str">
-        <v>+1h21min</v>
+        <v>+9h26min</v>
       </c>
       <c r="D48">
-        <v>81</v>
+        <v>566</v>
       </c>
     </row>
     <row r="49">
@@ -1082,13 +1076,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B49" t="str">
-        <v>Raquele Fragoso Da Silva</v>
+        <v>Maria Victoria Souza Araujo Ferro</v>
       </c>
       <c r="C49" t="str">
-        <v>-35h27min</v>
+        <v>-29h32min</v>
       </c>
       <c r="D49">
-        <v>-2127</v>
+        <v>-1772</v>
       </c>
     </row>
     <row r="50">
@@ -1096,41 +1090,41 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B50" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Marília Alice dos Santos Silva</v>
       </c>
       <c r="C50" t="str">
-        <v>-2h59min</v>
+        <v>+1h21min</v>
       </c>
       <c r="D50">
-        <v>-179</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B51" t="str">
-        <v>Eduarda Pereira Costa Silva</v>
+        <v>Raquele Fragoso Da Silva</v>
       </c>
       <c r="C51" t="str">
-        <v>+0h37min</v>
+        <v>-35h27min</v>
       </c>
       <c r="D51">
-        <v>37</v>
+        <v>-2127</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B52" t="str">
-        <v>Gabrielle Vitoria dos Santos</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
       <c r="C52" t="str">
-        <v>-6h23min</v>
+        <v>-2h59min</v>
       </c>
       <c r="D52">
-        <v>-383</v>
+        <v>-179</v>
       </c>
     </row>
     <row r="53">
@@ -1138,13 +1132,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B53" t="str">
-        <v>Larissa Alexia da Silva Souza</v>
+        <v>Eduarda Pereira Costa Silva</v>
       </c>
       <c r="C53" t="str">
-        <v>-3h32min</v>
+        <v>+0h37min</v>
       </c>
       <c r="D53">
-        <v>-212</v>
+        <v>37</v>
       </c>
     </row>
     <row r="54">
@@ -1152,13 +1146,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B54" t="str">
-        <v>Maria Cicília Brito Veiga</v>
+        <v>Larissa Alexia da Silva Souza</v>
       </c>
       <c r="C54" t="str">
-        <v>-3h41min</v>
+        <v>-3h32min</v>
       </c>
       <c r="D54">
-        <v>-221</v>
+        <v>-212</v>
       </c>
     </row>
     <row r="55">
@@ -1166,13 +1160,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B55" t="str">
-        <v>Maryanna Francielly Trajano da Silva</v>
+        <v>Maria Cicília Brito Veiga</v>
       </c>
       <c r="C55" t="str">
-        <v>-18h50min</v>
+        <v>-3h41min</v>
       </c>
       <c r="D55">
-        <v>-1130</v>
+        <v>-221</v>
       </c>
     </row>
     <row r="56">
@@ -1180,13 +1174,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B56" t="str">
-        <v>Robéria Gilo Da Silva</v>
+        <v>Maryanna Francielly Trajano da Silva</v>
       </c>
       <c r="C56" t="str">
-        <v>+53h25min</v>
+        <v>-18h50min</v>
       </c>
       <c r="D56">
-        <v>3205</v>
+        <v>-1130</v>
       </c>
     </row>
     <row r="57">
@@ -1197,10 +1191,10 @@
         <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
       <c r="C57" t="str">
-        <v>+19h52min</v>
+        <v>+19h32min</v>
       </c>
       <c r="D57">
-        <v>1192</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="58">
@@ -1267,10 +1261,10 @@
         <v>Camille Kauane Da Silva Nunes</v>
       </c>
       <c r="C62" t="str">
-        <v>+4h59min</v>
+        <v>+6h23min</v>
       </c>
       <c r="D62">
-        <v>299</v>
+        <v>383</v>
       </c>
     </row>
     <row r="63">
@@ -1572,13 +1566,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B84" t="str">
-        <v>Leidiane Souza</v>
+        <v>Joanna Roberta de Queiroz Viana</v>
       </c>
       <c r="C84" t="str">
-        <v>-4896h</v>
+        <v>+0h</v>
       </c>
       <c r="D84">
-        <v>-293760</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1586,7 +1580,7 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B85" t="str">
-        <v>Luiz Henrique Martins Tavares</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="C85" t="str">
         <v>-4896h</v>
@@ -1600,13 +1594,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B86" t="str">
-        <v>Maria Jeane da Silva Santos</v>
+        <v>Luiz Henrique Martins Tavares</v>
       </c>
       <c r="C86" t="str">
-        <v>+2h59min</v>
+        <v>-4896h</v>
       </c>
       <c r="D86">
-        <v>179</v>
+        <v>-293760</v>
       </c>
     </row>
     <row r="87">

</xml_diff>

<commit_message>
Atualiza dados - 12/04/2026 14:19
</commit_message>
<xml_diff>
--- a/public/saldo_por_gestor.xlsx
+++ b/public/saldo_por_gestor.xlsx
@@ -981,10 +981,10 @@
         <v>Bruna Candido de Lima</v>
       </c>
       <c r="C42" t="str">
-        <v>+3h37min</v>
+        <v>+4h58min</v>
       </c>
       <c r="D42">
-        <v>217</v>
+        <v>298</v>
       </c>
     </row>
     <row r="43">
@@ -995,10 +995,10 @@
         <v>Camilla Emanuelle Lopes de Almeida</v>
       </c>
       <c r="C43" t="str">
-        <v>-9h21min</v>
+        <v>-5h16min</v>
       </c>
       <c r="D43">
-        <v>-561</v>
+        <v>-316</v>
       </c>
     </row>
     <row r="44">
@@ -1009,10 +1009,10 @@
         <v>Danielle Dos Santos Silva</v>
       </c>
       <c r="C44" t="str">
-        <v>-26h55min</v>
+        <v>-14h56min</v>
       </c>
       <c r="D44">
-        <v>-1615</v>
+        <v>-896</v>
       </c>
     </row>
     <row r="45">
@@ -1023,10 +1023,10 @@
         <v>Edna Lopes Da Silva</v>
       </c>
       <c r="C45" t="str">
-        <v>+12h</v>
+        <v>+13h26min</v>
       </c>
       <c r="D45">
-        <v>720</v>
+        <v>806</v>
       </c>
     </row>
     <row r="46">
@@ -1037,10 +1037,10 @@
         <v>Jordelle Meygre Costa De Oliveira</v>
       </c>
       <c r="C46" t="str">
-        <v>+25h47min</v>
+        <v>+21h47min</v>
       </c>
       <c r="D46">
-        <v>1547</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="47">
@@ -1051,10 +1051,10 @@
         <v>Lays da Silva Vieira</v>
       </c>
       <c r="C47" t="str">
-        <v>+0h27min</v>
+        <v>+9h5min</v>
       </c>
       <c r="D47">
-        <v>27</v>
+        <v>545</v>
       </c>
     </row>
     <row r="48">
@@ -1065,10 +1065,10 @@
         <v>Luan Santos de Oliveira</v>
       </c>
       <c r="C48" t="str">
-        <v>+9h26min</v>
+        <v>+8h20min</v>
       </c>
       <c r="D48">
-        <v>566</v>
+        <v>500</v>
       </c>
     </row>
     <row r="49">
@@ -1079,10 +1079,10 @@
         <v>Maria Victoria Souza Araujo Ferro</v>
       </c>
       <c r="C49" t="str">
-        <v>-29h32min</v>
+        <v>-19h29min</v>
       </c>
       <c r="D49">
-        <v>-1772</v>
+        <v>-1169</v>
       </c>
     </row>
     <row r="50">
@@ -1093,10 +1093,10 @@
         <v>Marília Alice dos Santos Silva</v>
       </c>
       <c r="C50" t="str">
-        <v>+1h21min</v>
+        <v>+6h23min</v>
       </c>
       <c r="D50">
-        <v>81</v>
+        <v>383</v>
       </c>
     </row>
     <row r="51">
@@ -1121,10 +1121,10 @@
         <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
       <c r="C52" t="str">
-        <v>-2h59min</v>
+        <v>+0h41min</v>
       </c>
       <c r="D52">
-        <v>-179</v>
+        <v>41</v>
       </c>
     </row>
     <row r="53">

</xml_diff>

<commit_message>
Atualiza dados - 13/04/2026 15:40
</commit_message>
<xml_diff>
--- a/public/saldo_por_gestor.xlsx
+++ b/public/saldo_por_gestor.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D95"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -656,13 +656,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B19" t="str">
-        <v>Anny Karoline Andrade Santos</v>
+        <v>Kamilla Santos da Silva</v>
       </c>
       <c r="C19" t="str">
-        <v>-44h19min</v>
+        <v>-23h12min</v>
       </c>
       <c r="D19">
-        <v>-2659</v>
+        <v>-1392</v>
       </c>
     </row>
     <row r="20">
@@ -670,13 +670,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B20" t="str">
-        <v>Kamilla Santos da Silva</v>
+        <v>Maria Jeane da Silva Santos</v>
       </c>
       <c r="C20" t="str">
-        <v>-23h12min</v>
+        <v>+2h59min</v>
       </c>
       <c r="D20">
-        <v>-1392</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21">
@@ -684,13 +684,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B21" t="str">
-        <v>Maria Jeane da Silva Santos</v>
+        <v>Rodrigo Augusto Teixeira Dos Santos</v>
       </c>
       <c r="C21" t="str">
-        <v>+2h59min</v>
+        <v>+20h3min</v>
       </c>
       <c r="D21">
-        <v>179</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="22">
@@ -698,13 +698,13 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B22" t="str">
-        <v>Rodrigo Augusto Teixeira Dos Santos</v>
+        <v>Sandra da Conceição Freitas</v>
       </c>
       <c r="C22" t="str">
-        <v>+20h3min</v>
+        <v>+5h6min</v>
       </c>
       <c r="D22">
-        <v>1203</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23">
@@ -712,41 +712,41 @@
         <v>Ana Clara de Matos Chagas</v>
       </c>
       <c r="B23" t="str">
-        <v>Sandra da Conceição Freitas</v>
+        <v>Thamires Emanuelle da Silva</v>
       </c>
       <c r="C23" t="str">
-        <v>+5h6min</v>
+        <v>-2h26min</v>
       </c>
       <c r="D23">
-        <v>306</v>
+        <v>-146</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Ana Clara de Matos Chagas</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="B24" t="str">
-        <v>Thamires Emanuelle da Silva</v>
+        <v>Carlos Eduardo Silva De Oliveira</v>
       </c>
       <c r="C24" t="str">
-        <v>-2h26min</v>
+        <v>-61h48min</v>
       </c>
       <c r="D24">
-        <v>-146</v>
+        <v>-3708</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B25" t="str">
-        <v>Carlos Eduardo Silva De Oliveira</v>
+        <v>Ana Luiza Dos Santos</v>
       </c>
       <c r="C25" t="str">
-        <v>-61h48min</v>
+        <v>-19h20min</v>
       </c>
       <c r="D25">
-        <v>-3708</v>
+        <v>-1160</v>
       </c>
     </row>
     <row r="26">
@@ -754,13 +754,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B26" t="str">
-        <v>Ana Luiza Dos Santos</v>
+        <v>Emanoelle Feitosa Vieira Santos</v>
       </c>
       <c r="C26" t="str">
-        <v>-29h7min</v>
+        <v>-31h57min</v>
       </c>
       <c r="D26">
-        <v>-1747</v>
+        <v>-1917</v>
       </c>
     </row>
     <row r="27">
@@ -768,13 +768,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B27" t="str">
-        <v>Emanoelle Feitosa Vieira Santos</v>
+        <v>Gessica Aparecida Dos Santos</v>
       </c>
       <c r="C27" t="str">
-        <v>-31h57min</v>
+        <v>-96h27min</v>
       </c>
       <c r="D27">
-        <v>-1917</v>
+        <v>-5787</v>
       </c>
     </row>
     <row r="28">
@@ -782,13 +782,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B28" t="str">
-        <v>Gessica Aparecida Dos Santos</v>
+        <v>Giselle Dos Santos Roberto</v>
       </c>
       <c r="C28" t="str">
-        <v>-96h27min</v>
+        <v>-47h7min</v>
       </c>
       <c r="D28">
-        <v>-5787</v>
+        <v>-2827</v>
       </c>
     </row>
     <row r="29">
@@ -796,13 +796,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B29" t="str">
-        <v>Giselle Dos Santos Roberto</v>
+        <v>Kauanne Iwashita Da Silva</v>
       </c>
       <c r="C29" t="str">
-        <v>-47h7min</v>
+        <v>-32h13min</v>
       </c>
       <c r="D29">
-        <v>-2827</v>
+        <v>-1933</v>
       </c>
     </row>
     <row r="30">
@@ -810,13 +810,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B30" t="str">
-        <v>Kauanne Iwashita Da Silva</v>
+        <v>Laís Manuelle Santos Pereira</v>
       </c>
       <c r="C30" t="str">
-        <v>-32h13min</v>
+        <v>-16h57min</v>
       </c>
       <c r="D30">
-        <v>-1933</v>
+        <v>-1017</v>
       </c>
     </row>
     <row r="31">
@@ -824,13 +824,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B31" t="str">
-        <v>Laís Manuelle Santos Pereira</v>
+        <v>Leticia Seixas Santos</v>
       </c>
       <c r="C31" t="str">
-        <v>-16h57min</v>
+        <v>-12h19min</v>
       </c>
       <c r="D31">
-        <v>-1017</v>
+        <v>-739</v>
       </c>
     </row>
     <row r="32">
@@ -838,13 +838,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B32" t="str">
-        <v>Leticia Seixas Santos</v>
+        <v>Luciene Da Silva Nascimento</v>
       </c>
       <c r="C32" t="str">
-        <v>-12h19min</v>
+        <v>-39h36min</v>
       </c>
       <c r="D32">
-        <v>-739</v>
+        <v>-2376</v>
       </c>
     </row>
     <row r="33">
@@ -852,13 +852,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B33" t="str">
-        <v>Luciene Da Silva Nascimento</v>
+        <v>Natali de Souza Gonzaga</v>
       </c>
       <c r="C33" t="str">
-        <v>-39h36min</v>
+        <v>-52h14min</v>
       </c>
       <c r="D33">
-        <v>-2376</v>
+        <v>-3134</v>
       </c>
     </row>
     <row r="34">
@@ -866,13 +866,13 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B34" t="str">
-        <v>Natali de Souza Gonzaga</v>
+        <v>Nathalia Vieira Lima</v>
       </c>
       <c r="C34" t="str">
-        <v>-58h39min</v>
+        <v>-68h15min</v>
       </c>
       <c r="D34">
-        <v>-3519</v>
+        <v>-4095</v>
       </c>
     </row>
     <row r="35">
@@ -880,27 +880,27 @@
         <v>Erick Café Santos Júnior</v>
       </c>
       <c r="B35" t="str">
-        <v>Nathalia Vieira Lima</v>
+        <v>Sabrina Domingos Santos</v>
       </c>
       <c r="C35" t="str">
-        <v>-73h26min</v>
+        <v>+0h</v>
       </c>
       <c r="D35">
-        <v>-4406</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Erick Café Santos Júnior</v>
+        <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B36" t="str">
-        <v>Sabrina Domingos Santos</v>
+        <v>Fabia Batista da Silva</v>
       </c>
       <c r="C36" t="str">
-        <v>+0h</v>
+        <v>-26h19min</v>
       </c>
       <c r="D36">
-        <v>0</v>
+        <v>-1579</v>
       </c>
     </row>
     <row r="37">
@@ -908,13 +908,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B37" t="str">
-        <v>Fabia Batista da Silva</v>
+        <v>Gessyca Nayara Rocha Santos</v>
       </c>
       <c r="C37" t="str">
-        <v>-26h19min</v>
+        <v>-43h12min</v>
       </c>
       <c r="D37">
-        <v>-1579</v>
+        <v>-2592</v>
       </c>
     </row>
     <row r="38">
@@ -922,13 +922,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B38" t="str">
-        <v>Gessyca Nayara Rocha Santos</v>
+        <v>Jaine Mariana Rodrigues Mendonça</v>
       </c>
       <c r="C38" t="str">
-        <v>-43h12min</v>
+        <v>-3h42min</v>
       </c>
       <c r="D38">
-        <v>-2592</v>
+        <v>-222</v>
       </c>
     </row>
     <row r="39">
@@ -936,13 +936,13 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B39" t="str">
-        <v>Jaine Mariana Rodrigues Mendonça</v>
+        <v>Karine Celestino Evangelista dos Santos</v>
       </c>
       <c r="C39" t="str">
-        <v>-3h42min</v>
+        <v>-12h53min</v>
       </c>
       <c r="D39">
-        <v>-222</v>
+        <v>-773</v>
       </c>
     </row>
     <row r="40">
@@ -950,27 +950,27 @@
         <v>Joao Antonio Tavares Santos</v>
       </c>
       <c r="B40" t="str">
-        <v>Karine Celestino Evangelista dos Santos</v>
+        <v>Maria Tatiane Oliveira Santos</v>
       </c>
       <c r="C40" t="str">
-        <v>-12h53min</v>
+        <v>-52h59min</v>
       </c>
       <c r="D40">
-        <v>-773</v>
+        <v>-3179</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Joao Antonio Tavares Santos</v>
+        <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B41" t="str">
-        <v>Maria Tatiane Oliveira Santos</v>
+        <v>Bruna Candido de Lima</v>
       </c>
       <c r="C41" t="str">
-        <v>-52h59min</v>
+        <v>+4h58min</v>
       </c>
       <c r="D41">
-        <v>-3179</v>
+        <v>298</v>
       </c>
     </row>
     <row r="42">
@@ -978,13 +978,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B42" t="str">
-        <v>Bruna Candido de Lima</v>
+        <v>Camilla Emanuelle Lopes de Almeida</v>
       </c>
       <c r="C42" t="str">
-        <v>+4h58min</v>
+        <v>-5h16min</v>
       </c>
       <c r="D42">
-        <v>298</v>
+        <v>-316</v>
       </c>
     </row>
     <row r="43">
@@ -992,13 +992,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B43" t="str">
-        <v>Camilla Emanuelle Lopes de Almeida</v>
+        <v>Danielle Dos Santos Silva</v>
       </c>
       <c r="C43" t="str">
-        <v>-5h16min</v>
+        <v>-14h56min</v>
       </c>
       <c r="D43">
-        <v>-316</v>
+        <v>-896</v>
       </c>
     </row>
     <row r="44">
@@ -1006,13 +1006,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B44" t="str">
-        <v>Danielle Dos Santos Silva</v>
+        <v>Edna Lopes Da Silva</v>
       </c>
       <c r="C44" t="str">
-        <v>-14h56min</v>
+        <v>+13h26min</v>
       </c>
       <c r="D44">
-        <v>-896</v>
+        <v>806</v>
       </c>
     </row>
     <row r="45">
@@ -1020,13 +1020,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B45" t="str">
-        <v>Edna Lopes Da Silva</v>
+        <v>Jordelle Meygre Costa De Oliveira</v>
       </c>
       <c r="C45" t="str">
-        <v>+13h26min</v>
+        <v>+21h47min</v>
       </c>
       <c r="D45">
-        <v>806</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="46">
@@ -1034,13 +1034,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B46" t="str">
-        <v>Jordelle Meygre Costa De Oliveira</v>
+        <v>Lays da Silva Vieira</v>
       </c>
       <c r="C46" t="str">
-        <v>+21h47min</v>
+        <v>+9h5min</v>
       </c>
       <c r="D46">
-        <v>1307</v>
+        <v>545</v>
       </c>
     </row>
     <row r="47">
@@ -1048,13 +1048,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B47" t="str">
-        <v>Lays da Silva Vieira</v>
+        <v>Luan Santos de Oliveira</v>
       </c>
       <c r="C47" t="str">
-        <v>+9h5min</v>
+        <v>+8h20min</v>
       </c>
       <c r="D47">
-        <v>545</v>
+        <v>500</v>
       </c>
     </row>
     <row r="48">
@@ -1062,13 +1062,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B48" t="str">
-        <v>Luan Santos de Oliveira</v>
+        <v>Maria Victoria Souza Araujo Ferro</v>
       </c>
       <c r="C48" t="str">
-        <v>+8h20min</v>
+        <v>-19h29min</v>
       </c>
       <c r="D48">
-        <v>500</v>
+        <v>-1169</v>
       </c>
     </row>
     <row r="49">
@@ -1076,13 +1076,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B49" t="str">
-        <v>Maria Victoria Souza Araujo Ferro</v>
+        <v>Marília Alice dos Santos Silva</v>
       </c>
       <c r="C49" t="str">
-        <v>-19h29min</v>
+        <v>+10h25min</v>
       </c>
       <c r="D49">
-        <v>-1169</v>
+        <v>625</v>
       </c>
     </row>
     <row r="50">
@@ -1090,13 +1090,13 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B50" t="str">
-        <v>Marília Alice dos Santos Silva</v>
+        <v>Raquele Fragoso Da Silva</v>
       </c>
       <c r="C50" t="str">
-        <v>+6h23min</v>
+        <v>-35h27min</v>
       </c>
       <c r="D50">
-        <v>383</v>
+        <v>-2127</v>
       </c>
     </row>
     <row r="51">
@@ -1104,27 +1104,27 @@
         <v>Jonathan Henrique da Conceição Silva</v>
       </c>
       <c r="B51" t="str">
-        <v>Raquele Fragoso Da Silva</v>
+        <v>Yasmim Da Rocha Bezerra Barbosa</v>
       </c>
       <c r="C51" t="str">
-        <v>-35h27min</v>
+        <v>+0h41min</v>
       </c>
       <c r="D51">
-        <v>-2127</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Jonathan Henrique da Conceição Silva</v>
+        <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B52" t="str">
-        <v>Yasmim Da Rocha Bezerra Barbosa</v>
+        <v>Eduarda Pereira Costa Silva</v>
       </c>
       <c r="C52" t="str">
-        <v>+0h41min</v>
+        <v>+0h37min</v>
       </c>
       <c r="D52">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="53">
@@ -1132,13 +1132,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B53" t="str">
-        <v>Eduarda Pereira Costa Silva</v>
+        <v>Larissa Alexia da Silva Souza</v>
       </c>
       <c r="C53" t="str">
-        <v>+0h37min</v>
+        <v>-3h32min</v>
       </c>
       <c r="D53">
-        <v>37</v>
+        <v>-212</v>
       </c>
     </row>
     <row r="54">
@@ -1146,13 +1146,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B54" t="str">
-        <v>Larissa Alexia da Silva Souza</v>
+        <v>Maria Cicília Brito Veiga</v>
       </c>
       <c r="C54" t="str">
-        <v>-3h32min</v>
+        <v>-3h41min</v>
       </c>
       <c r="D54">
-        <v>-212</v>
+        <v>-221</v>
       </c>
     </row>
     <row r="55">
@@ -1160,13 +1160,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B55" t="str">
-        <v>Maria Cicília Brito Veiga</v>
+        <v>Maryanna Francielly Trajano da Silva</v>
       </c>
       <c r="C55" t="str">
-        <v>-3h41min</v>
+        <v>-18h50min</v>
       </c>
       <c r="D55">
-        <v>-221</v>
+        <v>-1130</v>
       </c>
     </row>
     <row r="56">
@@ -1174,13 +1174,13 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B56" t="str">
-        <v>Maryanna Francielly Trajano da Silva</v>
+        <v>Valesca Meirelle Bezerra Vitória</v>
       </c>
       <c r="C56" t="str">
-        <v>-18h50min</v>
+        <v>+19h32min</v>
       </c>
       <c r="D56">
-        <v>-1130</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="57">
@@ -1188,41 +1188,41 @@
         <v>Kemilly Rafaelly Souza Silva</v>
       </c>
       <c r="B57" t="str">
-        <v>Valesca Meirelle Bezerra Vitória</v>
+        <v>Yasmin Abilia Ferro da Silva</v>
       </c>
       <c r="C57" t="str">
-        <v>+19h32min</v>
+        <v>+5h28min</v>
       </c>
       <c r="D57">
-        <v>1172</v>
+        <v>328</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Kemilly Rafaelly Souza Silva</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="B58" t="str">
-        <v>Yasmin Abilia Ferro da Silva</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="C58" t="str">
-        <v>+5h28min</v>
+        <v>-19h5min</v>
       </c>
       <c r="D58">
-        <v>328</v>
+        <v>-1145</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Leidiane Souza</v>
+        <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B59" t="str">
-        <v>Mariane Santos Sousa</v>
+        <v>Ana Paula Amaral Santos Ismerim</v>
       </c>
       <c r="C59" t="str">
-        <v>-19h5min</v>
+        <v>-28h34min</v>
       </c>
       <c r="D59">
-        <v>-1145</v>
+        <v>-1714</v>
       </c>
     </row>
     <row r="60">
@@ -1230,13 +1230,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B60" t="str">
-        <v>Ana Paula Amaral Santos Ismerim</v>
+        <v>Bruna Rayane Oliveira dos Santos</v>
       </c>
       <c r="C60" t="str">
-        <v>-28h34min</v>
+        <v>+7h13min</v>
       </c>
       <c r="D60">
-        <v>-1714</v>
+        <v>433</v>
       </c>
     </row>
     <row r="61">
@@ -1244,13 +1244,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B61" t="str">
-        <v>Bruna Rayane Oliveira dos Santos</v>
+        <v>Camille Kauane Da Silva Nunes</v>
       </c>
       <c r="C61" t="str">
-        <v>+7h13min</v>
+        <v>+6h23min</v>
       </c>
       <c r="D61">
-        <v>433</v>
+        <v>383</v>
       </c>
     </row>
     <row r="62">
@@ -1258,13 +1258,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B62" t="str">
-        <v>Camille Kauane Da Silva Nunes</v>
+        <v>Cristielle Pereira Lima Da Silva</v>
       </c>
       <c r="C62" t="str">
-        <v>+6h23min</v>
+        <v>-18h14min</v>
       </c>
       <c r="D62">
-        <v>383</v>
+        <v>-1094</v>
       </c>
     </row>
     <row r="63">
@@ -1272,13 +1272,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B63" t="str">
-        <v>Cristielle Pereira Lima Da Silva</v>
+        <v>Deise Gislaine Silva vitor</v>
       </c>
       <c r="C63" t="str">
-        <v>-18h14min</v>
+        <v>+22h59min</v>
       </c>
       <c r="D63">
-        <v>-1094</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="64">
@@ -1286,13 +1286,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B64" t="str">
-        <v>Deise Gislaine Silva vitor</v>
+        <v>Eliene Da Silva Santos</v>
       </c>
       <c r="C64" t="str">
-        <v>+22h59min</v>
+        <v>+85h10min</v>
       </c>
       <c r="D64">
-        <v>1379</v>
+        <v>5110</v>
       </c>
     </row>
     <row r="65">
@@ -1300,13 +1300,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B65" t="str">
-        <v>Eliene Da Silva Santos</v>
+        <v>Maria Tatiane Basto Cardoso</v>
       </c>
       <c r="C65" t="str">
-        <v>+85h10min</v>
+        <v>+56h4min</v>
       </c>
       <c r="D65">
-        <v>5110</v>
+        <v>3364</v>
       </c>
     </row>
     <row r="66">
@@ -1314,13 +1314,13 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B66" t="str">
-        <v>Maria Tatiane Basto Cardoso</v>
+        <v>Samyra Anchieta Bispo</v>
       </c>
       <c r="C66" t="str">
-        <v>+56h4min</v>
+        <v>-2h32min</v>
       </c>
       <c r="D66">
-        <v>3364</v>
+        <v>-152</v>
       </c>
     </row>
     <row r="67">
@@ -1328,27 +1328,27 @@
         <v>Maria Taciane Pereira Barbosa</v>
       </c>
       <c r="B67" t="str">
-        <v>Samyra Anchieta Bispo</v>
+        <v>THAMIRYS SILVESTRINI MORALES</v>
       </c>
       <c r="C67" t="str">
-        <v>-2h32min</v>
+        <v>-6h7min</v>
       </c>
       <c r="D67">
-        <v>-152</v>
+        <v>-367</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Maria Taciane Pereira Barbosa</v>
+        <v>Mariane Santos Sousa</v>
       </c>
       <c r="B68" t="str">
-        <v>THAMIRYS SILVESTRINI MORALES</v>
+        <v>Anny Karoline Andrade Santos</v>
       </c>
       <c r="C68" t="str">
-        <v>-6h7min</v>
+        <v>-44h19min</v>
       </c>
       <c r="D68">
-        <v>-367</v>
+        <v>-2659</v>
       </c>
     </row>
     <row r="69">
@@ -1580,13 +1580,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B85" t="str">
-        <v>Leidiane Souza</v>
+        <v>Josenildo Alves da silva Júnior</v>
       </c>
       <c r="C85" t="str">
-        <v>-4896h</v>
+        <v>+0h</v>
       </c>
       <c r="D85">
-        <v>-293760</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -1594,7 +1594,7 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B86" t="str">
-        <v>Luiz Henrique Martins Tavares</v>
+        <v>Leidiane Souza</v>
       </c>
       <c r="C86" t="str">
         <v>-4896h</v>
@@ -1608,13 +1608,13 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B87" t="str">
-        <v>Moises Santiago</v>
+        <v>Luiz Henrique Martins Tavares</v>
       </c>
       <c r="C87" t="str">
-        <v>-3148h</v>
+        <v>-4896h</v>
       </c>
       <c r="D87">
-        <v>-188880</v>
+        <v>-293760</v>
       </c>
     </row>
     <row r="88">
@@ -1622,7 +1622,7 @@
         <v>Sem Gestor</v>
       </c>
       <c r="B88" t="str">
-        <v>Paulo Rogério Santos</v>
+        <v>Maria Fernanda Gomes Vieira</v>
       </c>
       <c r="C88" t="str">
         <v>+0h</v>
@@ -1633,44 +1633,44 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B89" t="str">
-        <v>João Ricardo Dantas Albuquerque</v>
+        <v>Moises Santiago</v>
       </c>
       <c r="C89" t="str">
-        <v>-18h58min</v>
+        <v>-3148h</v>
       </c>
       <c r="D89">
-        <v>-1138</v>
+        <v>-188880</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B90" t="str">
-        <v>Lianda Melinda Santos Calixto</v>
+        <v>Paulo Rogério Santos</v>
       </c>
       <c r="C90" t="str">
-        <v>-23h48min</v>
+        <v>+0h</v>
       </c>
       <c r="D90">
-        <v>-1428</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Suzana Martins Tavares</v>
+        <v>Sem Gestor</v>
       </c>
       <c r="B91" t="str">
-        <v>Ravy Thiago Vieira Da Silva</v>
+        <v>Shayane Oliveira Ferreira</v>
       </c>
       <c r="C91" t="str">
-        <v>+27h35min</v>
+        <v>+0h</v>
       </c>
       <c r="D91">
-        <v>1655</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -1678,18 +1678,60 @@
         <v>Suzana Martins Tavares</v>
       </c>
       <c r="B92" t="str">
+        <v>João Ricardo Dantas Albuquerque</v>
+      </c>
+      <c r="C92" t="str">
+        <v>-18h58min</v>
+      </c>
+      <c r="D92">
+        <v>-1138</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Lianda Melinda Santos Calixto</v>
+      </c>
+      <c r="C93" t="str">
+        <v>-23h48min</v>
+      </c>
+      <c r="D93">
+        <v>-1428</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Ravy Thiago Vieira Da Silva</v>
+      </c>
+      <c r="C94" t="str">
+        <v>+27h35min</v>
+      </c>
+      <c r="D94">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Suzana Martins Tavares</v>
+      </c>
+      <c r="B95" t="str">
         <v>Thayane Mayara dos Santos</v>
       </c>
-      <c r="C92" t="str">
+      <c r="C95" t="str">
         <v>-64h4min</v>
       </c>
-      <c r="D92">
+      <c r="D95">
         <v>-3844</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D95"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>